<commit_message>
Custom supplier price & USB conn added in BOM.
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/eSpark-BOM(5 Boards).xlsx
+++ b/Deliverables/BOM/eSpark-BOM(5 Boards).xlsx
@@ -5,23 +5,24 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Melih-SoundSensor\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\Melih-SoundSensor\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F9320C6-7A10-4DD9-AEED-8F59393BD1A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7DCCF14-03CB-4DC0-922D-DC993A177CE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="171">
   <si>
     <t>S. No.</t>
   </si>
@@ -133,9 +134,6 @@
     <t>X1</t>
   </si>
   <si>
-    <t>Aliexpress</t>
-  </si>
-  <si>
     <t>J3</t>
   </si>
   <si>
@@ -383,12 +381,6 @@
   </si>
   <si>
     <t>3-644456-5</t>
-  </si>
-  <si>
-    <t>Surface Mount DC Power Receptacle 1.2mm 3.7mm SMD AC/DC Power Connectors ROHS</t>
-  </si>
-  <si>
-    <t>DC-0920-SMT</t>
   </si>
   <si>
     <t>2 PIN JST Connector</t>
@@ -513,12 +505,6 @@
 </t>
   </si>
   <si>
-    <t>XKB</t>
-  </si>
-  <si>
-    <t>C692456</t>
-  </si>
-  <si>
     <t>------</t>
   </si>
   <si>
@@ -545,6 +531,21 @@
   </si>
   <si>
     <t>Battery</t>
+  </si>
+  <si>
+    <t>Custom Supplier</t>
+  </si>
+  <si>
+    <t>10118194-0001LF</t>
+  </si>
+  <si>
+    <t>USB 2.0 1 5 Female Micro-B SMD USB Connectors ROHS</t>
+  </si>
+  <si>
+    <t>C132563</t>
+  </si>
+  <si>
+    <t>Amphenol ICC</t>
   </si>
 </sst>
 </file>
@@ -553,8 +554,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0000"/>
-    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="167" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
   </numFmts>
   <fonts count="26">
     <font>
@@ -1253,7 +1254,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="194">
+  <cellXfs count="195">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1287,19 +1288,19 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1321,18 +1322,6 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1348,19 +1337,10 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="14" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1375,39 +1355,431 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="7" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="7" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="165" fontId="9" fillId="7" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="20" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="7" borderId="20" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="7" borderId="17" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="26" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="30" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="24" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="28" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="22" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="7" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="11" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="7" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="11" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="7" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="26" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="9" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="24" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="4" borderId="24" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1416,11 +1788,13 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1429,396 +1803,26 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="19" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="20" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="7" borderId="20" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="7" borderId="17" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="26" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="30" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="24" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="28" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="22" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="7" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="11" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="7" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="11" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="7" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="26" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="9" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="24" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="4" borderId="24" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2102,7 +2106,7 @@
     <col min="1" max="1" width="6.140625" style="2" customWidth="1"/>
     <col min="2" max="2" width="14.42578125" style="1" customWidth="1"/>
     <col min="3" max="3" width="47.5703125" style="20" customWidth="1"/>
-    <col min="4" max="4" width="33.140625" style="31" customWidth="1"/>
+    <col min="4" max="4" width="33.140625" style="27" customWidth="1"/>
     <col min="5" max="5" width="21" style="2" customWidth="1"/>
     <col min="6" max="6" width="28.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -2112,7 +2116,7 @@
     <col min="11" max="11" width="14.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="21.85546875" style="1" customWidth="1"/>
     <col min="13" max="13" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17" style="1" customWidth="1"/>
     <col min="15" max="15" width="12.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -2121,26 +2125,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="16.5" thickBot="1">
-      <c r="A1" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
-      <c r="M1" s="27"/>
-      <c r="N1" s="27"/>
-      <c r="O1" s="27"/>
-      <c r="P1" s="27"/>
-      <c r="Q1" s="27"/>
-      <c r="R1" s="28"/>
+      <c r="A1" s="183" t="s">
+        <v>163</v>
+      </c>
+      <c r="B1" s="184"/>
+      <c r="C1" s="184"/>
+      <c r="D1" s="184"/>
+      <c r="E1" s="184"/>
+      <c r="F1" s="184"/>
+      <c r="G1" s="184"/>
+      <c r="H1" s="184"/>
+      <c r="I1" s="184"/>
+      <c r="J1" s="184"/>
+      <c r="K1" s="184"/>
+      <c r="L1" s="184"/>
+      <c r="M1" s="184"/>
+      <c r="N1" s="184"/>
+      <c r="O1" s="184"/>
+      <c r="P1" s="184"/>
+      <c r="Q1" s="184"/>
+      <c r="R1" s="185"/>
     </row>
     <row r="2" spans="1:19" ht="16.5" thickBot="1">
       <c r="A2" s="3" t="s">
@@ -2174,22 +2178,22 @@
         <v>9</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L2" s="5" t="s">
         <v>10</v>
       </c>
       <c r="M2" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="N2" s="5" t="s">
         <v>11</v>
       </c>
       <c r="O2" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="P2" s="5" t="s">
         <v>47</v>
-      </c>
-      <c r="P2" s="5" t="s">
-        <v>48</v>
       </c>
       <c r="Q2" s="5" t="s">
         <v>12</v>
@@ -2202,50 +2206,50 @@
       <c r="A3" s="6">
         <v>1</v>
       </c>
-      <c r="B3" s="34" t="s">
+      <c r="B3" s="190" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="129" t="s">
+      <c r="C3" s="115" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3" s="116" t="s">
         <v>50</v>
       </c>
-      <c r="D3" s="130" t="s">
+      <c r="E3" s="117" t="s">
         <v>51</v>
       </c>
-      <c r="E3" s="131" t="s">
+      <c r="F3" s="117" t="s">
         <v>52</v>
       </c>
-      <c r="F3" s="131" t="s">
-        <v>53</v>
-      </c>
-      <c r="G3" s="68" t="s">
-        <v>124</v>
-      </c>
-      <c r="H3" s="69" t="s">
-        <v>125</v>
-      </c>
-      <c r="I3" s="70" t="s">
-        <v>40</v>
-      </c>
-      <c r="J3" s="130" t="s">
+      <c r="G3" s="54" t="s">
+        <v>121</v>
+      </c>
+      <c r="H3" s="55" t="s">
+        <v>122</v>
+      </c>
+      <c r="I3" s="56" t="s">
+        <v>39</v>
+      </c>
+      <c r="J3" s="116" t="s">
         <v>20</v>
       </c>
-      <c r="K3" s="71">
+      <c r="K3" s="57">
         <v>20</v>
       </c>
-      <c r="L3" s="132">
+      <c r="L3" s="118">
         <v>3</v>
       </c>
-      <c r="M3" s="72">
+      <c r="M3" s="58">
         <f>L3*5</f>
         <v>15</v>
       </c>
-      <c r="N3" s="133" t="s">
+      <c r="N3" s="119" t="s">
         <v>16</v>
       </c>
-      <c r="O3" s="73">
+      <c r="O3" s="59">
         <v>2.58E-2</v>
       </c>
-      <c r="P3" s="74">
+      <c r="P3" s="60">
         <f>O3*K3</f>
         <v>0.51600000000000001</v>
       </c>
@@ -2256,48 +2260,48 @@
       <c r="A4" s="6">
         <v>2</v>
       </c>
-      <c r="B4" s="35"/>
-      <c r="C4" s="134" t="s">
+      <c r="B4" s="191"/>
+      <c r="C4" s="120" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="135" t="s">
+      <c r="D4" s="121" t="s">
+        <v>53</v>
+      </c>
+      <c r="E4" s="122" t="s">
+        <v>51</v>
+      </c>
+      <c r="F4" s="122" t="s">
         <v>54</v>
       </c>
-      <c r="E4" s="136" t="s">
-        <v>52</v>
-      </c>
-      <c r="F4" s="136" t="s">
-        <v>55</v>
-      </c>
-      <c r="G4" s="75" t="s">
-        <v>124</v>
-      </c>
-      <c r="H4" s="76" t="s">
-        <v>126</v>
-      </c>
-      <c r="I4" s="77" t="s">
-        <v>40</v>
-      </c>
-      <c r="J4" s="135" t="s">
-        <v>73</v>
-      </c>
-      <c r="K4" s="78">
+      <c r="G4" s="61" t="s">
+        <v>121</v>
+      </c>
+      <c r="H4" s="62" t="s">
+        <v>123</v>
+      </c>
+      <c r="I4" s="63" t="s">
+        <v>39</v>
+      </c>
+      <c r="J4" s="121" t="s">
+        <v>72</v>
+      </c>
+      <c r="K4" s="64">
         <v>20</v>
       </c>
-      <c r="L4" s="137">
+      <c r="L4" s="123">
         <v>1</v>
       </c>
-      <c r="M4" s="79">
+      <c r="M4" s="65">
         <f t="shared" ref="M4:M27" si="0">L4*5</f>
         <v>5</v>
       </c>
-      <c r="N4" s="138" t="s">
+      <c r="N4" s="124" t="s">
         <v>16</v>
       </c>
-      <c r="O4" s="80">
+      <c r="O4" s="66">
         <v>2.0299999999999999E-2</v>
       </c>
-      <c r="P4" s="81">
+      <c r="P4" s="67">
         <f t="shared" ref="P4:P25" si="1">O4*K4</f>
         <v>0.40599999999999997</v>
       </c>
@@ -2308,48 +2312,48 @@
       <c r="A5" s="6">
         <v>3</v>
       </c>
-      <c r="B5" s="35"/>
-      <c r="C5" s="134" t="s">
+      <c r="B5" s="191"/>
+      <c r="C5" s="120" t="s">
+        <v>55</v>
+      </c>
+      <c r="D5" s="125" t="s">
         <v>56</v>
       </c>
-      <c r="D5" s="139" t="s">
+      <c r="E5" s="121" t="s">
+        <v>51</v>
+      </c>
+      <c r="F5" s="121" t="s">
         <v>57</v>
       </c>
-      <c r="E5" s="135" t="s">
-        <v>52</v>
-      </c>
-      <c r="F5" s="135" t="s">
-        <v>58</v>
-      </c>
-      <c r="G5" s="82" t="s">
-        <v>127</v>
-      </c>
-      <c r="H5" s="76" t="s">
-        <v>128</v>
-      </c>
-      <c r="I5" s="77" t="s">
-        <v>40</v>
-      </c>
-      <c r="J5" s="135" t="s">
+      <c r="G5" s="68" t="s">
+        <v>124</v>
+      </c>
+      <c r="H5" s="62" t="s">
+        <v>125</v>
+      </c>
+      <c r="I5" s="63" t="s">
+        <v>39</v>
+      </c>
+      <c r="J5" s="121" t="s">
         <v>15</v>
       </c>
-      <c r="K5" s="78">
+      <c r="K5" s="64">
         <v>100</v>
       </c>
-      <c r="L5" s="137">
+      <c r="L5" s="123">
         <v>15</v>
       </c>
-      <c r="M5" s="79">
+      <c r="M5" s="65">
         <f t="shared" si="0"/>
         <v>75</v>
       </c>
-      <c r="N5" s="138" t="s">
+      <c r="N5" s="124" t="s">
         <v>16</v>
       </c>
-      <c r="O5" s="80">
+      <c r="O5" s="66">
         <v>7.3000000000000001E-3</v>
       </c>
-      <c r="P5" s="81">
+      <c r="P5" s="67">
         <f t="shared" si="1"/>
         <v>0.73</v>
       </c>
@@ -2361,48 +2365,48 @@
       <c r="A6" s="6">
         <v>4</v>
       </c>
-      <c r="B6" s="35"/>
-      <c r="C6" s="134" t="s">
+      <c r="B6" s="191"/>
+      <c r="C6" s="120" t="s">
+        <v>58</v>
+      </c>
+      <c r="D6" s="121" t="s">
         <v>59</v>
       </c>
-      <c r="D6" s="135" t="s">
+      <c r="E6" s="122" t="s">
         <v>60</v>
       </c>
-      <c r="E6" s="136" t="s">
+      <c r="F6" s="122" t="s">
         <v>61</v>
       </c>
-      <c r="F6" s="136" t="s">
-        <v>62</v>
-      </c>
-      <c r="G6" s="82" t="s">
-        <v>127</v>
-      </c>
-      <c r="H6" s="76" t="s">
-        <v>129</v>
-      </c>
-      <c r="I6" s="77" t="s">
-        <v>40</v>
-      </c>
-      <c r="J6" s="135" t="s">
-        <v>74</v>
-      </c>
-      <c r="K6" s="78">
+      <c r="G6" s="68" t="s">
+        <v>124</v>
+      </c>
+      <c r="H6" s="62" t="s">
+        <v>126</v>
+      </c>
+      <c r="I6" s="63" t="s">
+        <v>39</v>
+      </c>
+      <c r="J6" s="121" t="s">
+        <v>73</v>
+      </c>
+      <c r="K6" s="64">
         <v>100</v>
       </c>
-      <c r="L6" s="137">
+      <c r="L6" s="123">
         <v>8</v>
       </c>
-      <c r="M6" s="79">
+      <c r="M6" s="65">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="N6" s="140" t="s">
+      <c r="N6" s="126" t="s">
         <v>16</v>
       </c>
-      <c r="O6" s="80">
+      <c r="O6" s="66">
         <v>3.7000000000000002E-3</v>
       </c>
-      <c r="P6" s="81">
+      <c r="P6" s="67">
         <f t="shared" si="1"/>
         <v>0.37</v>
       </c>
@@ -2414,52 +2418,52 @@
       <c r="A7" s="6">
         <v>5</v>
       </c>
-      <c r="B7" s="35"/>
-      <c r="C7" s="134" t="s">
+      <c r="B7" s="191"/>
+      <c r="C7" s="120" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="139" t="s">
-        <v>63</v>
-      </c>
-      <c r="E7" s="135" t="s">
-        <v>52</v>
-      </c>
-      <c r="F7" s="135" t="s">
+      <c r="D7" s="125" t="s">
+        <v>62</v>
+      </c>
+      <c r="E7" s="121" t="s">
+        <v>51</v>
+      </c>
+      <c r="F7" s="121" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="82" t="s">
+      <c r="G7" s="68" t="s">
+        <v>124</v>
+      </c>
+      <c r="H7" s="62" t="s">
         <v>127</v>
       </c>
-      <c r="H7" s="76" t="s">
-        <v>130</v>
-      </c>
-      <c r="I7" s="77" t="s">
-        <v>40</v>
-      </c>
-      <c r="J7" s="135" t="s">
+      <c r="I7" s="63" t="s">
+        <v>39</v>
+      </c>
+      <c r="J7" s="121" t="s">
         <v>19</v>
       </c>
-      <c r="K7" s="78">
+      <c r="K7" s="64">
         <v>150</v>
       </c>
-      <c r="L7" s="137">
+      <c r="L7" s="123">
         <v>24</v>
       </c>
-      <c r="M7" s="79">
+      <c r="M7" s="65">
         <f t="shared" si="0"/>
         <v>120</v>
       </c>
-      <c r="N7" s="140" t="s">
+      <c r="N7" s="126" t="s">
         <v>16</v>
       </c>
-      <c r="O7" s="80">
+      <c r="O7" s="66">
         <v>7.9000000000000008E-3</v>
       </c>
-      <c r="P7" s="81">
+      <c r="P7" s="67">
         <f t="shared" si="1"/>
         <v>1.1850000000000001</v>
       </c>
-      <c r="Q7" s="37"/>
+      <c r="Q7" s="30"/>
       <c r="R7" s="15"/>
       <c r="S7" s="11"/>
     </row>
@@ -2467,48 +2471,48 @@
       <c r="A8" s="6">
         <v>6</v>
       </c>
-      <c r="B8" s="35"/>
-      <c r="C8" s="134" t="s">
+      <c r="B8" s="191"/>
+      <c r="C8" s="120" t="s">
+        <v>63</v>
+      </c>
+      <c r="D8" s="121" t="s">
         <v>64</v>
       </c>
-      <c r="D8" s="135" t="s">
+      <c r="E8" s="122" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" s="122" t="s">
         <v>65</v>
       </c>
-      <c r="E8" s="136" t="s">
-        <v>52</v>
-      </c>
-      <c r="F8" s="136" t="s">
-        <v>66</v>
-      </c>
-      <c r="G8" s="82" t="s">
-        <v>131</v>
-      </c>
-      <c r="H8" s="83" t="s">
-        <v>132</v>
-      </c>
-      <c r="I8" s="77" t="s">
-        <v>40</v>
-      </c>
-      <c r="J8" s="135" t="s">
-        <v>75</v>
-      </c>
-      <c r="K8" s="82">
+      <c r="G8" s="68" t="s">
+        <v>128</v>
+      </c>
+      <c r="H8" s="69" t="s">
+        <v>129</v>
+      </c>
+      <c r="I8" s="63" t="s">
+        <v>39</v>
+      </c>
+      <c r="J8" s="121" t="s">
+        <v>74</v>
+      </c>
+      <c r="K8" s="68">
         <v>10</v>
       </c>
-      <c r="L8" s="137">
+      <c r="L8" s="123">
         <v>1</v>
       </c>
-      <c r="M8" s="79">
+      <c r="M8" s="65">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N8" s="140" t="s">
+      <c r="N8" s="126" t="s">
         <v>16</v>
       </c>
-      <c r="O8" s="80">
+      <c r="O8" s="66">
         <v>4.4299999999999999E-2</v>
       </c>
-      <c r="P8" s="81">
+      <c r="P8" s="67">
         <f t="shared" si="1"/>
         <v>0.443</v>
       </c>
@@ -2520,48 +2524,48 @@
       <c r="A9" s="6">
         <v>7</v>
       </c>
-      <c r="B9" s="35"/>
-      <c r="C9" s="134" t="s">
+      <c r="B9" s="191"/>
+      <c r="C9" s="120" t="s">
+        <v>66</v>
+      </c>
+      <c r="D9" s="121" t="s">
         <v>67</v>
       </c>
-      <c r="D9" s="135" t="s">
+      <c r="E9" s="122" t="s">
+        <v>51</v>
+      </c>
+      <c r="F9" s="122" t="s">
         <v>68</v>
       </c>
-      <c r="E9" s="136" t="s">
-        <v>52</v>
-      </c>
-      <c r="F9" s="136" t="s">
-        <v>69</v>
-      </c>
-      <c r="G9" s="82" t="s">
-        <v>127</v>
-      </c>
-      <c r="H9" s="76" t="s">
-        <v>133</v>
-      </c>
-      <c r="I9" s="77" t="s">
-        <v>40</v>
-      </c>
-      <c r="J9" s="135" t="s">
-        <v>76</v>
-      </c>
-      <c r="K9" s="82">
+      <c r="G9" s="68" t="s">
+        <v>124</v>
+      </c>
+      <c r="H9" s="62" t="s">
+        <v>130</v>
+      </c>
+      <c r="I9" s="63" t="s">
+        <v>39</v>
+      </c>
+      <c r="J9" s="121" t="s">
+        <v>75</v>
+      </c>
+      <c r="K9" s="68">
         <v>100</v>
       </c>
-      <c r="L9" s="137">
+      <c r="L9" s="123">
         <v>6</v>
       </c>
-      <c r="M9" s="79">
+      <c r="M9" s="65">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="N9" s="138" t="s">
+      <c r="N9" s="124" t="s">
         <v>16</v>
       </c>
-      <c r="O9" s="80">
+      <c r="O9" s="66">
         <v>3.2000000000000002E-3</v>
       </c>
-      <c r="P9" s="81">
+      <c r="P9" s="67">
         <f t="shared" si="1"/>
         <v>0.32</v>
       </c>
@@ -2573,268 +2577,268 @@
       <c r="A10" s="6">
         <v>8</v>
       </c>
-      <c r="B10" s="36"/>
-      <c r="C10" s="141" t="s">
+      <c r="B10" s="192"/>
+      <c r="C10" s="127" t="s">
+        <v>69</v>
+      </c>
+      <c r="D10" s="128" t="s">
         <v>70</v>
       </c>
-      <c r="D10" s="142" t="s">
+      <c r="E10" s="129" t="s">
+        <v>51</v>
+      </c>
+      <c r="F10" s="129" t="s">
         <v>71</v>
       </c>
-      <c r="E10" s="143" t="s">
-        <v>52</v>
-      </c>
-      <c r="F10" s="143" t="s">
-        <v>72</v>
-      </c>
-      <c r="G10" s="84" t="s">
-        <v>127</v>
-      </c>
-      <c r="H10" s="85" t="s">
-        <v>134</v>
-      </c>
-      <c r="I10" s="86" t="s">
-        <v>40</v>
-      </c>
-      <c r="J10" s="143" t="s">
-        <v>77</v>
-      </c>
-      <c r="K10" s="84">
+      <c r="G10" s="70" t="s">
+        <v>124</v>
+      </c>
+      <c r="H10" s="71" t="s">
+        <v>131</v>
+      </c>
+      <c r="I10" s="72" t="s">
+        <v>39</v>
+      </c>
+      <c r="J10" s="129" t="s">
+        <v>76</v>
+      </c>
+      <c r="K10" s="70">
         <v>100</v>
       </c>
-      <c r="L10" s="144">
+      <c r="L10" s="130">
         <v>16</v>
       </c>
-      <c r="M10" s="87">
+      <c r="M10" s="73">
         <f t="shared" si="0"/>
         <v>80</v>
       </c>
-      <c r="N10" s="145" t="s">
+      <c r="N10" s="131" t="s">
         <v>16</v>
       </c>
-      <c r="O10" s="88">
+      <c r="O10" s="74">
         <v>1.7299999999999999E-2</v>
       </c>
-      <c r="P10" s="89">
+      <c r="P10" s="75">
         <f t="shared" si="1"/>
         <v>1.73</v>
       </c>
-      <c r="Q10" s="42"/>
-      <c r="R10" s="43"/>
+      <c r="Q10" s="35"/>
+      <c r="R10" s="36"/>
       <c r="S10" s="11"/>
     </row>
     <row r="11" spans="1:19" ht="26.25" thickBot="1">
       <c r="A11" s="6">
         <v>9</v>
       </c>
-      <c r="B11" s="40" t="s">
-        <v>81</v>
-      </c>
-      <c r="C11" s="146" t="s">
+      <c r="B11" s="33" t="s">
+        <v>80</v>
+      </c>
+      <c r="C11" s="132" t="s">
+        <v>77</v>
+      </c>
+      <c r="D11" s="133" t="s">
         <v>78</v>
       </c>
-      <c r="D11" s="147" t="s">
+      <c r="E11" s="134" t="s">
+        <v>28</v>
+      </c>
+      <c r="F11" s="134" t="s">
         <v>79</v>
       </c>
-      <c r="E11" s="148" t="s">
-        <v>28</v>
-      </c>
-      <c r="F11" s="148" t="s">
-        <v>80</v>
-      </c>
-      <c r="G11" s="90" t="s">
-        <v>164</v>
-      </c>
-      <c r="H11" s="91" t="s">
-        <v>162</v>
-      </c>
-      <c r="I11" s="92" t="s">
-        <v>163</v>
-      </c>
-      <c r="J11" s="93" t="s">
+      <c r="G11" s="76" t="s">
+        <v>159</v>
+      </c>
+      <c r="H11" s="77" t="s">
+        <v>157</v>
+      </c>
+      <c r="I11" s="78" t="s">
+        <v>158</v>
+      </c>
+      <c r="J11" s="79" t="s">
         <v>22</v>
       </c>
-      <c r="K11" s="93">
+      <c r="K11" s="79">
         <v>42</v>
       </c>
-      <c r="L11" s="94">
+      <c r="L11" s="80">
         <v>8</v>
       </c>
-      <c r="M11" s="94">
+      <c r="M11" s="80">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="N11" s="149" t="s">
-        <v>34</v>
-      </c>
-      <c r="O11" s="95">
-        <v>6.5</v>
-      </c>
-      <c r="P11" s="96">
+      <c r="N11" s="135" t="s">
+        <v>166</v>
+      </c>
+      <c r="O11" s="81">
+        <v>3.68</v>
+      </c>
+      <c r="P11" s="82">
         <f t="shared" si="1"/>
-        <v>273</v>
-      </c>
-      <c r="Q11" s="49" t="s">
-        <v>149</v>
-      </c>
-      <c r="R11" s="50"/>
+        <v>154.56</v>
+      </c>
+      <c r="Q11" s="42" t="s">
+        <v>146</v>
+      </c>
+      <c r="R11" s="43"/>
       <c r="S11" s="11"/>
     </row>
     <row r="12" spans="1:19" ht="26.25" thickBot="1">
       <c r="A12" s="6">
         <v>10</v>
       </c>
-      <c r="B12" s="40" t="s">
+      <c r="B12" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="150" t="s">
+      <c r="C12" s="136" t="s">
+        <v>81</v>
+      </c>
+      <c r="D12" s="137" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="138" t="s">
+        <v>28</v>
+      </c>
+      <c r="F12" s="138" t="s">
         <v>82</v>
       </c>
-      <c r="D12" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="152" t="s">
-        <v>28</v>
-      </c>
-      <c r="F12" s="152" t="s">
-        <v>83</v>
-      </c>
-      <c r="G12" s="97" t="s">
-        <v>135</v>
-      </c>
-      <c r="H12" s="98" t="s">
-        <v>136</v>
-      </c>
-      <c r="I12" s="99" t="s">
-        <v>40</v>
-      </c>
-      <c r="J12" s="100" t="s">
+      <c r="G12" s="83" t="s">
+        <v>132</v>
+      </c>
+      <c r="H12" s="84" t="s">
+        <v>133</v>
+      </c>
+      <c r="I12" s="85" t="s">
+        <v>39</v>
+      </c>
+      <c r="J12" s="86" t="s">
         <v>22</v>
       </c>
-      <c r="K12" s="100">
+      <c r="K12" s="86">
         <v>10</v>
       </c>
-      <c r="L12" s="101">
+      <c r="L12" s="87">
         <v>1</v>
       </c>
-      <c r="M12" s="101">
+      <c r="M12" s="87">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N12" s="153" t="s">
+      <c r="N12" s="139" t="s">
         <v>16</v>
       </c>
-      <c r="O12" s="102">
+      <c r="O12" s="88">
         <v>6.0600000000000001E-2</v>
       </c>
-      <c r="P12" s="103">
+      <c r="P12" s="89">
         <f t="shared" si="1"/>
         <v>0.60599999999999998</v>
       </c>
-      <c r="Q12" s="41"/>
-      <c r="R12" s="48"/>
+      <c r="Q12" s="34"/>
+      <c r="R12" s="41"/>
       <c r="S12" s="11"/>
     </row>
     <row r="13" spans="1:19" ht="26.25" thickBot="1">
       <c r="A13" s="6">
         <v>11</v>
       </c>
-      <c r="B13" s="34" t="s">
+      <c r="B13" s="190" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="154" t="s">
+      <c r="C13" s="140" t="s">
+        <v>83</v>
+      </c>
+      <c r="D13" s="141" t="s">
+        <v>33</v>
+      </c>
+      <c r="E13" s="141" t="s">
+        <v>28</v>
+      </c>
+      <c r="F13" s="141" t="s">
         <v>84</v>
       </c>
-      <c r="D13" s="155" t="s">
-        <v>33</v>
-      </c>
-      <c r="E13" s="155" t="s">
-        <v>28</v>
-      </c>
-      <c r="F13" s="155" t="s">
-        <v>85</v>
-      </c>
-      <c r="G13" s="104" t="s">
-        <v>137</v>
-      </c>
-      <c r="H13" s="105" t="s">
-        <v>138</v>
-      </c>
-      <c r="I13" s="106" t="s">
-        <v>40</v>
-      </c>
-      <c r="J13" s="107" t="s">
+      <c r="G13" s="90" t="s">
+        <v>134</v>
+      </c>
+      <c r="H13" s="91" t="s">
+        <v>135</v>
+      </c>
+      <c r="I13" s="92" t="s">
+        <v>39</v>
+      </c>
+      <c r="J13" s="93" t="s">
         <v>22</v>
       </c>
-      <c r="K13" s="107">
+      <c r="K13" s="93">
         <v>7</v>
       </c>
-      <c r="L13" s="108">
+      <c r="L13" s="94">
         <v>1</v>
       </c>
-      <c r="M13" s="108">
+      <c r="M13" s="94">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N13" s="156" t="s">
+      <c r="N13" s="142" t="s">
         <v>16</v>
       </c>
-      <c r="O13" s="109">
+      <c r="O13" s="95">
         <v>0.25650000000000001</v>
       </c>
-      <c r="P13" s="110">
-        <f t="shared" si="1"/>
+      <c r="P13" s="96">
+        <f>O13*K13</f>
         <v>1.7955000000000001</v>
       </c>
       <c r="Q13" s="18"/>
-      <c r="R13" s="51"/>
+      <c r="R13" s="44"/>
       <c r="S13" s="11"/>
     </row>
     <row r="14" spans="1:19" ht="26.25" thickBot="1">
       <c r="A14" s="6">
         <v>12</v>
       </c>
-      <c r="B14" s="36"/>
-      <c r="C14" s="157" t="s">
+      <c r="B14" s="192"/>
+      <c r="C14" s="143" t="s">
+        <v>85</v>
+      </c>
+      <c r="D14" s="144" t="s">
         <v>86</v>
       </c>
-      <c r="D14" s="158" t="s">
+      <c r="E14" s="145" t="s">
+        <v>28</v>
+      </c>
+      <c r="F14" s="145" t="s">
         <v>87</v>
       </c>
-      <c r="E14" s="159" t="s">
-        <v>28</v>
-      </c>
-      <c r="F14" s="159" t="s">
-        <v>88</v>
-      </c>
-      <c r="G14" s="111" t="s">
-        <v>139</v>
-      </c>
-      <c r="H14" s="112" t="s">
-        <v>140</v>
-      </c>
-      <c r="I14" s="113" t="s">
-        <v>40</v>
-      </c>
-      <c r="J14" s="114" t="s">
+      <c r="G14" s="97" t="s">
+        <v>136</v>
+      </c>
+      <c r="H14" s="98" t="s">
+        <v>137</v>
+      </c>
+      <c r="I14" s="99" t="s">
+        <v>39</v>
+      </c>
+      <c r="J14" s="100" t="s">
         <v>22</v>
       </c>
-      <c r="K14" s="114">
+      <c r="K14" s="100">
         <v>7</v>
       </c>
-      <c r="L14" s="115">
+      <c r="L14" s="101">
         <v>2</v>
       </c>
-      <c r="M14" s="101">
+      <c r="M14" s="87">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="N14" s="160" t="s">
+      <c r="N14" s="146" t="s">
         <v>16</v>
       </c>
-      <c r="O14" s="116">
+      <c r="O14" s="102">
         <v>0.1215</v>
       </c>
-      <c r="P14" s="103">
+      <c r="P14" s="89">
         <f t="shared" si="1"/>
         <v>0.85050000000000003</v>
       </c>
@@ -2846,50 +2850,50 @@
       <c r="A15" s="6">
         <v>13</v>
       </c>
-      <c r="B15" s="34" t="s">
+      <c r="B15" s="190" t="s">
         <v>23</v>
       </c>
-      <c r="C15" s="154" t="s">
+      <c r="C15" s="140" t="s">
+        <v>88</v>
+      </c>
+      <c r="D15" s="141" t="s">
         <v>89</v>
       </c>
-      <c r="D15" s="155" t="s">
+      <c r="E15" s="116" t="s">
+        <v>24</v>
+      </c>
+      <c r="F15" s="147" t="s">
         <v>90</v>
       </c>
-      <c r="E15" s="130" t="s">
-        <v>24</v>
-      </c>
-      <c r="F15" s="161" t="s">
-        <v>91</v>
-      </c>
-      <c r="G15" s="68" t="s">
-        <v>143</v>
-      </c>
-      <c r="H15" s="69" t="s">
-        <v>142</v>
-      </c>
-      <c r="I15" s="117" t="s">
-        <v>141</v>
-      </c>
-      <c r="J15" s="130" t="s">
-        <v>95</v>
-      </c>
-      <c r="K15" s="118">
+      <c r="G15" s="54" t="s">
+        <v>140</v>
+      </c>
+      <c r="H15" s="55" t="s">
+        <v>139</v>
+      </c>
+      <c r="I15" s="103" t="s">
+        <v>138</v>
+      </c>
+      <c r="J15" s="116" t="s">
+        <v>94</v>
+      </c>
+      <c r="K15" s="104">
         <v>100</v>
       </c>
-      <c r="L15" s="118">
+      <c r="L15" s="104">
         <v>2</v>
       </c>
-      <c r="M15" s="72">
+      <c r="M15" s="58">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="N15" s="162" t="s">
+      <c r="N15" s="148" t="s">
         <v>16</v>
       </c>
-      <c r="O15" s="73">
+      <c r="O15" s="59">
         <v>1E-3</v>
       </c>
-      <c r="P15" s="74">
+      <c r="P15" s="60">
         <f t="shared" si="1"/>
         <v>0.1</v>
       </c>
@@ -2901,48 +2905,48 @@
       <c r="A16" s="6">
         <v>14</v>
       </c>
-      <c r="B16" s="36"/>
-      <c r="C16" s="157" t="s">
+      <c r="B16" s="192"/>
+      <c r="C16" s="143" t="s">
+        <v>91</v>
+      </c>
+      <c r="D16" s="144" t="s">
         <v>92</v>
       </c>
-      <c r="D16" s="158" t="s">
+      <c r="E16" s="145" t="s">
+        <v>24</v>
+      </c>
+      <c r="F16" s="145" t="s">
         <v>93</v>
       </c>
-      <c r="E16" s="159" t="s">
-        <v>24</v>
-      </c>
-      <c r="F16" s="159" t="s">
-        <v>94</v>
-      </c>
-      <c r="G16" s="111" t="s">
-        <v>127</v>
-      </c>
-      <c r="H16" s="112" t="s">
-        <v>144</v>
-      </c>
-      <c r="I16" s="113" t="s">
-        <v>40</v>
-      </c>
-      <c r="J16" s="159" t="s">
+      <c r="G16" s="97" t="s">
+        <v>124</v>
+      </c>
+      <c r="H16" s="98" t="s">
+        <v>141</v>
+      </c>
+      <c r="I16" s="99" t="s">
+        <v>39</v>
+      </c>
+      <c r="J16" s="145" t="s">
         <v>25</v>
       </c>
-      <c r="K16" s="119">
+      <c r="K16" s="105">
         <v>100</v>
       </c>
-      <c r="L16" s="119">
+      <c r="L16" s="105">
         <v>1</v>
       </c>
-      <c r="M16" s="101">
+      <c r="M16" s="87">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N16" s="163" t="s">
+      <c r="N16" s="149" t="s">
         <v>16</v>
       </c>
-      <c r="O16" s="116">
+      <c r="O16" s="102">
         <v>1.4E-3</v>
       </c>
-      <c r="P16" s="103">
+      <c r="P16" s="89">
         <f t="shared" si="1"/>
         <v>0.13999999999999999</v>
       </c>
@@ -2954,50 +2958,50 @@
       <c r="A17" s="6">
         <v>15</v>
       </c>
-      <c r="B17" s="34" t="s">
-        <v>115</v>
-      </c>
-      <c r="C17" s="154" t="s">
+      <c r="B17" s="190" t="s">
+        <v>114</v>
+      </c>
+      <c r="C17" s="140" t="s">
+        <v>95</v>
+      </c>
+      <c r="D17" s="141" t="s">
         <v>96</v>
       </c>
-      <c r="D17" s="155" t="s">
+      <c r="E17" s="116" t="s">
         <v>97</v>
       </c>
-      <c r="E17" s="130" t="s">
+      <c r="F17" s="116" t="s">
         <v>98</v>
       </c>
-      <c r="F17" s="130" t="s">
-        <v>99</v>
-      </c>
-      <c r="G17" s="68" t="s">
+      <c r="G17" s="54" t="s">
         <v>31</v>
       </c>
-      <c r="H17" s="69" t="s">
-        <v>145</v>
-      </c>
-      <c r="I17" s="70" t="s">
-        <v>40</v>
-      </c>
-      <c r="J17" s="71" t="s">
+      <c r="H17" s="55" t="s">
+        <v>142</v>
+      </c>
+      <c r="I17" s="56" t="s">
+        <v>39</v>
+      </c>
+      <c r="J17" s="57" t="s">
         <v>22</v>
       </c>
-      <c r="K17" s="71">
+      <c r="K17" s="57">
         <v>11</v>
       </c>
-      <c r="L17" s="132">
+      <c r="L17" s="118">
         <v>2</v>
       </c>
-      <c r="M17" s="72">
+      <c r="M17" s="58">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="N17" s="164" t="s">
+      <c r="N17" s="150" t="s">
         <v>16</v>
       </c>
-      <c r="O17" s="73">
+      <c r="O17" s="59">
         <v>0.44729999999999998</v>
       </c>
-      <c r="P17" s="74">
+      <c r="P17" s="60">
         <f t="shared" si="1"/>
         <v>4.9203000000000001</v>
       </c>
@@ -3009,48 +3013,48 @@
       <c r="A18" s="6">
         <v>16</v>
       </c>
-      <c r="B18" s="35"/>
-      <c r="C18" s="165" t="s">
+      <c r="B18" s="191"/>
+      <c r="C18" s="151" t="s">
+        <v>99</v>
+      </c>
+      <c r="D18" s="125" t="s">
+        <v>30</v>
+      </c>
+      <c r="E18" s="121" t="s">
         <v>100</v>
       </c>
-      <c r="D18" s="139" t="s">
-        <v>30</v>
-      </c>
-      <c r="E18" s="135" t="s">
+      <c r="F18" s="121" t="s">
         <v>101</v>
       </c>
-      <c r="F18" s="135" t="s">
-        <v>102</v>
-      </c>
-      <c r="G18" s="77" t="s">
-        <v>146</v>
-      </c>
-      <c r="H18" s="77" t="s">
-        <v>147</v>
-      </c>
-      <c r="I18" s="77" t="s">
-        <v>40</v>
-      </c>
-      <c r="J18" s="78" t="s">
+      <c r="G18" s="63" t="s">
+        <v>143</v>
+      </c>
+      <c r="H18" s="63" t="s">
+        <v>144</v>
+      </c>
+      <c r="I18" s="63" t="s">
+        <v>39</v>
+      </c>
+      <c r="J18" s="64" t="s">
         <v>22</v>
       </c>
-      <c r="K18" s="77">
+      <c r="K18" s="63">
         <v>6</v>
       </c>
-      <c r="L18" s="137">
+      <c r="L18" s="123">
         <v>1</v>
       </c>
-      <c r="M18" s="79">
+      <c r="M18" s="65">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N18" s="140" t="s">
+      <c r="N18" s="126" t="s">
         <v>16</v>
       </c>
-      <c r="O18" s="80">
+      <c r="O18" s="66">
         <v>0.53200000000000003</v>
       </c>
-      <c r="P18" s="81">
+      <c r="P18" s="67">
         <f t="shared" si="1"/>
         <v>3.1920000000000002</v>
       </c>
@@ -3062,150 +3066,154 @@
       <c r="A19" s="6">
         <v>17</v>
       </c>
-      <c r="B19" s="35"/>
-      <c r="C19" s="165" t="s">
+      <c r="B19" s="191"/>
+      <c r="C19" s="151" t="s">
+        <v>102</v>
+      </c>
+      <c r="D19" s="125" t="s">
+        <v>29</v>
+      </c>
+      <c r="E19" s="121" t="s">
         <v>103</v>
       </c>
-      <c r="D19" s="139" t="s">
-        <v>29</v>
-      </c>
-      <c r="E19" s="135" t="s">
+      <c r="F19" s="121" t="s">
         <v>104</v>
       </c>
-      <c r="F19" s="135" t="s">
-        <v>105</v>
-      </c>
-      <c r="G19" s="82" t="s">
+      <c r="G19" s="68" t="s">
         <v>31</v>
       </c>
-      <c r="H19" s="82" t="s">
+      <c r="H19" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="I19" s="78" t="s">
-        <v>40</v>
-      </c>
-      <c r="J19" s="78" t="s">
+      <c r="I19" s="64" t="s">
+        <v>39</v>
+      </c>
+      <c r="J19" s="64" t="s">
         <v>22</v>
       </c>
-      <c r="K19" s="82">
+      <c r="K19" s="68">
         <v>6</v>
       </c>
-      <c r="L19" s="137">
+      <c r="L19" s="123">
         <v>1</v>
       </c>
-      <c r="M19" s="79">
+      <c r="M19" s="65">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N19" s="166" t="s">
-        <v>148</v>
-      </c>
-      <c r="O19" s="120">
+      <c r="N19" s="152" t="s">
+        <v>145</v>
+      </c>
+      <c r="O19" s="106">
         <v>8</v>
       </c>
-      <c r="P19" s="81">
+      <c r="P19" s="67">
         <f t="shared" si="1"/>
         <v>48</v>
       </c>
-      <c r="Q19" s="47" t="s">
-        <v>149</v>
-      </c>
-      <c r="R19" s="44"/>
+      <c r="Q19" s="40" t="s">
+        <v>146</v>
+      </c>
+      <c r="R19" s="37"/>
       <c r="S19" s="11"/>
     </row>
     <row r="20" spans="1:19" ht="15.75" thickBot="1">
       <c r="A20" s="6">
         <v>18</v>
       </c>
-      <c r="B20" s="35"/>
-      <c r="C20" s="175" t="s">
+      <c r="B20" s="191"/>
+      <c r="C20" s="161" t="s">
+        <v>105</v>
+      </c>
+      <c r="D20" s="162" t="s">
         <v>106</v>
       </c>
-      <c r="D20" s="176" t="s">
+      <c r="E20" s="163" t="s">
+        <v>147</v>
+      </c>
+      <c r="F20" s="163" t="s">
         <v>107</v>
       </c>
-      <c r="E20" s="177" t="s">
-        <v>150</v>
-      </c>
-      <c r="F20" s="177" t="s">
-        <v>108</v>
-      </c>
-      <c r="G20" s="178" t="s">
+      <c r="G20" s="164" t="s">
         <v>31</v>
       </c>
-      <c r="H20" s="178" t="s">
+      <c r="H20" s="164" t="s">
         <v>22</v>
       </c>
-      <c r="I20" s="177" t="s">
-        <v>40</v>
-      </c>
-      <c r="J20" s="177" t="s">
+      <c r="I20" s="163" t="s">
+        <v>39</v>
+      </c>
+      <c r="J20" s="163" t="s">
         <v>22</v>
       </c>
-      <c r="K20" s="178"/>
-      <c r="L20" s="179">
+      <c r="K20" s="164"/>
+      <c r="L20" s="165">
         <v>2</v>
       </c>
-      <c r="M20" s="180">
+      <c r="M20" s="166">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="N20" s="181"/>
-      <c r="O20" s="182"/>
-      <c r="P20" s="183">
+      <c r="N20" s="167" t="s">
+        <v>166</v>
+      </c>
+      <c r="O20" s="193">
+        <v>10.18</v>
+      </c>
+      <c r="P20" s="168">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="Q20" s="184"/>
-      <c r="R20" s="185"/>
+      <c r="Q20" s="169"/>
+      <c r="R20" s="170"/>
       <c r="S20" s="11"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1">
       <c r="A21" s="6">
         <v>19</v>
       </c>
-      <c r="B21" s="35"/>
-      <c r="C21" s="165" t="s">
+      <c r="B21" s="191"/>
+      <c r="C21" s="151" t="s">
+        <v>108</v>
+      </c>
+      <c r="D21" s="125" t="s">
         <v>109</v>
       </c>
-      <c r="D21" s="139" t="s">
+      <c r="E21" s="121" t="s">
+        <v>28</v>
+      </c>
+      <c r="F21" s="121" t="s">
         <v>110</v>
       </c>
-      <c r="E21" s="135" t="s">
-        <v>28</v>
-      </c>
-      <c r="F21" s="135" t="s">
-        <v>111</v>
-      </c>
-      <c r="G21" s="82" t="s">
-        <v>151</v>
-      </c>
-      <c r="H21" s="82" t="s">
-        <v>152</v>
-      </c>
-      <c r="I21" s="78" t="s">
-        <v>40</v>
-      </c>
-      <c r="J21" s="78" t="s">
+      <c r="G21" s="68" t="s">
+        <v>148</v>
+      </c>
+      <c r="H21" s="68" t="s">
+        <v>149</v>
+      </c>
+      <c r="I21" s="64" t="s">
+        <v>39</v>
+      </c>
+      <c r="J21" s="64" t="s">
         <v>22</v>
       </c>
-      <c r="K21" s="82">
+      <c r="K21" s="68">
         <v>6</v>
       </c>
-      <c r="L21" s="137">
+      <c r="L21" s="123">
         <v>1</v>
       </c>
-      <c r="M21" s="79">
+      <c r="M21" s="65">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N21" s="166" t="s">
+      <c r="N21" s="152" t="s">
         <v>16</v>
       </c>
-      <c r="O21" s="80">
+      <c r="O21" s="66">
         <v>4.1349999999999998</v>
       </c>
-      <c r="P21" s="81">
+      <c r="P21" s="67">
         <f t="shared" si="1"/>
         <v>24.81</v>
       </c>
@@ -3217,48 +3225,48 @@
       <c r="A22" s="6">
         <v>20</v>
       </c>
-      <c r="B22" s="36"/>
-      <c r="C22" s="157" t="s">
+      <c r="B22" s="192"/>
+      <c r="C22" s="143" t="s">
+        <v>111</v>
+      </c>
+      <c r="D22" s="144" t="s">
         <v>112</v>
       </c>
-      <c r="D22" s="158" t="s">
+      <c r="E22" s="145" t="s">
+        <v>150</v>
+      </c>
+      <c r="F22" s="145" t="s">
         <v>113</v>
       </c>
-      <c r="E22" s="159" t="s">
-        <v>153</v>
-      </c>
-      <c r="F22" s="159" t="s">
-        <v>114</v>
-      </c>
-      <c r="G22" s="114" t="s">
-        <v>154</v>
-      </c>
-      <c r="H22" s="114" t="s">
-        <v>155</v>
-      </c>
-      <c r="I22" s="114" t="s">
-        <v>40</v>
-      </c>
-      <c r="J22" s="114" t="s">
+      <c r="G22" s="100" t="s">
+        <v>151</v>
+      </c>
+      <c r="H22" s="100" t="s">
+        <v>152</v>
+      </c>
+      <c r="I22" s="100" t="s">
+        <v>39</v>
+      </c>
+      <c r="J22" s="100" t="s">
         <v>22</v>
       </c>
-      <c r="K22" s="111">
+      <c r="K22" s="97">
         <v>10</v>
       </c>
-      <c r="L22" s="167">
+      <c r="L22" s="153">
         <v>1</v>
       </c>
-      <c r="M22" s="101">
+      <c r="M22" s="87">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N22" s="168" t="s">
+      <c r="N22" s="154" t="s">
         <v>16</v>
       </c>
-      <c r="O22" s="116">
+      <c r="O22" s="102">
         <v>5.8799999999999998E-2</v>
       </c>
-      <c r="P22" s="103">
+      <c r="P22" s="89">
         <f t="shared" si="1"/>
         <v>0.58799999999999997</v>
       </c>
@@ -3270,50 +3278,50 @@
       <c r="A23" s="6">
         <v>21</v>
       </c>
-      <c r="B23" s="34" t="s">
-        <v>123</v>
-      </c>
-      <c r="C23" s="154" t="s">
+      <c r="B23" s="190" t="s">
+        <v>120</v>
+      </c>
+      <c r="C23" s="140" t="s">
+        <v>115</v>
+      </c>
+      <c r="D23" s="141" t="s">
+        <v>41</v>
+      </c>
+      <c r="E23" s="116" t="s">
+        <v>28</v>
+      </c>
+      <c r="F23" s="147" t="s">
         <v>116</v>
       </c>
-      <c r="D23" s="155" t="s">
-        <v>42</v>
-      </c>
-      <c r="E23" s="130" t="s">
-        <v>28</v>
-      </c>
-      <c r="F23" s="161" t="s">
-        <v>117</v>
-      </c>
-      <c r="G23" s="72" t="s">
-        <v>156</v>
-      </c>
-      <c r="H23" s="72" t="s">
-        <v>157</v>
-      </c>
-      <c r="I23" s="71" t="s">
-        <v>40</v>
-      </c>
-      <c r="J23" s="71" t="s">
+      <c r="G23" s="58" t="s">
+        <v>153</v>
+      </c>
+      <c r="H23" s="58" t="s">
+        <v>154</v>
+      </c>
+      <c r="I23" s="57" t="s">
+        <v>39</v>
+      </c>
+      <c r="J23" s="57" t="s">
         <v>22</v>
       </c>
-      <c r="K23" s="121">
+      <c r="K23" s="107">
         <v>50</v>
       </c>
-      <c r="L23" s="122">
+      <c r="L23" s="108">
         <v>1</v>
       </c>
-      <c r="M23" s="72">
+      <c r="M23" s="58">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N23" s="169" t="s">
+      <c r="N23" s="155" t="s">
         <v>16</v>
       </c>
-      <c r="O23" s="73">
+      <c r="O23" s="59">
         <v>1.5699999999999999E-2</v>
       </c>
-      <c r="P23" s="74">
+      <c r="P23" s="60">
         <f t="shared" si="1"/>
         <v>0.78499999999999992</v>
       </c>
@@ -3321,52 +3329,56 @@
       <c r="R23" s="13"/>
       <c r="S23" s="11"/>
     </row>
-    <row r="24" spans="1:19" ht="26.25" thickBot="1">
+    <row r="24" spans="1:19" ht="15.75" thickBot="1">
       <c r="A24" s="6">
         <v>22</v>
       </c>
-      <c r="B24" s="35"/>
-      <c r="C24" s="165" t="s">
-        <v>118</v>
-      </c>
-      <c r="D24" s="139" t="s">
-        <v>43</v>
-      </c>
-      <c r="E24" s="135" t="s">
+      <c r="B24" s="191"/>
+      <c r="C24" s="151" t="s">
+        <v>168</v>
+      </c>
+      <c r="D24" s="125" t="s">
+        <v>42</v>
+      </c>
+      <c r="E24" s="121" t="s">
         <v>28</v>
       </c>
-      <c r="F24" s="135" t="s">
-        <v>119</v>
-      </c>
-      <c r="G24" s="78" t="s">
-        <v>160</v>
-      </c>
-      <c r="H24" s="78" t="s">
-        <v>161</v>
-      </c>
-      <c r="I24" s="78" t="s">
-        <v>40</v>
-      </c>
-      <c r="J24" s="78" t="s">
+      <c r="F24" s="121" t="s">
+        <v>167</v>
+      </c>
+      <c r="G24" s="64" t="s">
+        <v>170</v>
+      </c>
+      <c r="H24" s="64" t="s">
+        <v>169</v>
+      </c>
+      <c r="I24" s="64" t="s">
+        <v>39</v>
+      </c>
+      <c r="J24" s="64" t="s">
         <v>22</v>
       </c>
-      <c r="K24" s="78">
+      <c r="K24" s="64">
         <v>6</v>
       </c>
-      <c r="L24" s="123">
+      <c r="L24" s="109">
         <v>1</v>
       </c>
-      <c r="M24" s="79">
+      <c r="M24" s="65">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N24" s="166"/>
-      <c r="O24" s="120"/>
-      <c r="P24" s="81">
+      <c r="N24" s="194" t="s">
+        <v>16</v>
+      </c>
+      <c r="O24" s="106">
+        <v>0.25409999999999999</v>
+      </c>
+      <c r="P24" s="67">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Q24" s="38"/>
+        <v>1.5246</v>
+      </c>
+      <c r="Q24" s="31"/>
       <c r="R24" s="15"/>
       <c r="S24" s="11"/>
     </row>
@@ -3374,52 +3386,52 @@
       <c r="A25" s="6">
         <v>23</v>
       </c>
-      <c r="B25" s="35"/>
-      <c r="C25" s="165" t="s">
-        <v>120</v>
-      </c>
-      <c r="D25" s="139" t="s">
-        <v>35</v>
-      </c>
-      <c r="E25" s="135" t="s">
+      <c r="B25" s="191"/>
+      <c r="C25" s="151" t="s">
+        <v>117</v>
+      </c>
+      <c r="D25" s="125" t="s">
+        <v>34</v>
+      </c>
+      <c r="E25" s="121" t="s">
         <v>28</v>
       </c>
-      <c r="F25" s="170" t="s">
-        <v>121</v>
-      </c>
-      <c r="G25" s="78" t="s">
-        <v>158</v>
-      </c>
-      <c r="H25" s="78" t="s">
-        <v>159</v>
-      </c>
-      <c r="I25" s="78" t="s">
-        <v>166</v>
-      </c>
-      <c r="J25" s="78" t="s">
+      <c r="F25" s="156" t="s">
+        <v>118</v>
+      </c>
+      <c r="G25" s="64" t="s">
+        <v>155</v>
+      </c>
+      <c r="H25" s="64" t="s">
+        <v>156</v>
+      </c>
+      <c r="I25" s="64" t="s">
+        <v>161</v>
+      </c>
+      <c r="J25" s="64" t="s">
         <v>22</v>
       </c>
-      <c r="K25" s="78">
+      <c r="K25" s="64">
         <v>50</v>
       </c>
-      <c r="L25" s="123">
+      <c r="L25" s="109">
         <v>1</v>
       </c>
-      <c r="M25" s="79">
+      <c r="M25" s="65">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N25" s="166" t="s">
+      <c r="N25" s="152" t="s">
         <v>16</v>
       </c>
-      <c r="O25" s="80">
+      <c r="O25" s="66">
         <v>1.26E-2</v>
       </c>
-      <c r="P25" s="81">
+      <c r="P25" s="67">
         <f t="shared" si="1"/>
         <v>0.63</v>
       </c>
-      <c r="Q25" s="39"/>
+      <c r="Q25" s="32"/>
       <c r="R25" s="15"/>
       <c r="S25" s="11"/>
     </row>
@@ -3427,107 +3439,107 @@
       <c r="A26" s="19">
         <v>24</v>
       </c>
-      <c r="B26" s="35"/>
-      <c r="C26" s="171" t="s">
+      <c r="B26" s="191"/>
+      <c r="C26" s="157" t="s">
+        <v>35</v>
+      </c>
+      <c r="D26" s="158" t="s">
+        <v>119</v>
+      </c>
+      <c r="E26" s="159" t="s">
         <v>36</v>
       </c>
-      <c r="D26" s="172" t="s">
-        <v>122</v>
-      </c>
-      <c r="E26" s="173" t="s">
-        <v>37</v>
-      </c>
-      <c r="F26" s="173" t="s">
-        <v>37</v>
-      </c>
-      <c r="G26" s="124" t="s">
-        <v>162</v>
-      </c>
-      <c r="H26" s="124" t="s">
-        <v>162</v>
-      </c>
-      <c r="I26" s="125" t="s">
-        <v>41</v>
-      </c>
-      <c r="J26" s="125" t="s">
-        <v>41</v>
-      </c>
-      <c r="K26" s="126" t="s">
-        <v>162</v>
-      </c>
-      <c r="L26" s="127">
+      <c r="F26" s="159" t="s">
+        <v>36</v>
+      </c>
+      <c r="G26" s="110" t="s">
+        <v>157</v>
+      </c>
+      <c r="H26" s="110" t="s">
+        <v>157</v>
+      </c>
+      <c r="I26" s="111" t="s">
+        <v>40</v>
+      </c>
+      <c r="J26" s="111" t="s">
+        <v>40</v>
+      </c>
+      <c r="K26" s="112" t="s">
+        <v>157</v>
+      </c>
+      <c r="L26" s="113">
         <v>42</v>
       </c>
-      <c r="M26" s="128">
+      <c r="M26" s="114">
         <f t="shared" si="0"/>
         <v>210</v>
       </c>
-      <c r="N26" s="124" t="s">
+      <c r="N26" s="110" t="s">
+        <v>157</v>
+      </c>
+      <c r="O26" s="111" t="s">
+        <v>40</v>
+      </c>
+      <c r="P26" s="112" t="s">
+        <v>157</v>
+      </c>
+      <c r="Q26" s="45" t="s">
         <v>162</v>
       </c>
-      <c r="O26" s="125" t="s">
-        <v>41</v>
-      </c>
-      <c r="P26" s="126" t="s">
-        <v>162</v>
-      </c>
-      <c r="Q26" s="52" t="s">
-        <v>167</v>
-      </c>
-      <c r="R26" s="53"/>
+      <c r="R26" s="46"/>
       <c r="S26" s="11"/>
     </row>
     <row r="27" spans="1:19" ht="15.75" thickBot="1">
       <c r="A27" s="19">
         <v>25</v>
       </c>
-      <c r="B27" s="174" t="s">
-        <v>169</v>
-      </c>
-      <c r="C27" s="186" t="s">
-        <v>170</v>
-      </c>
-      <c r="D27" s="193" t="s">
-        <v>41</v>
-      </c>
-      <c r="E27" s="193" t="s">
-        <v>41</v>
-      </c>
-      <c r="F27" s="187" t="s">
-        <v>170</v>
-      </c>
-      <c r="G27" s="193" t="s">
-        <v>41</v>
-      </c>
-      <c r="H27" s="193" t="s">
-        <v>41</v>
-      </c>
-      <c r="I27" s="193" t="s">
-        <v>41</v>
-      </c>
-      <c r="J27" s="193" t="s">
-        <v>41</v>
-      </c>
-      <c r="K27" s="193" t="s">
-        <v>41</v>
-      </c>
-      <c r="L27" s="190">
+      <c r="B27" s="160" t="s">
+        <v>164</v>
+      </c>
+      <c r="C27" s="171" t="s">
+        <v>165</v>
+      </c>
+      <c r="D27" s="178" t="s">
+        <v>40</v>
+      </c>
+      <c r="E27" s="178" t="s">
+        <v>40</v>
+      </c>
+      <c r="F27" s="172" t="s">
+        <v>165</v>
+      </c>
+      <c r="G27" s="178" t="s">
+        <v>40</v>
+      </c>
+      <c r="H27" s="178" t="s">
+        <v>40</v>
+      </c>
+      <c r="I27" s="178" t="s">
+        <v>40</v>
+      </c>
+      <c r="J27" s="178" t="s">
+        <v>40</v>
+      </c>
+      <c r="K27" s="178" t="s">
+        <v>40</v>
+      </c>
+      <c r="L27" s="175">
         <v>1</v>
       </c>
-      <c r="M27" s="190">
+      <c r="M27" s="175">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N27" s="188"/>
-      <c r="O27" s="189"/>
-      <c r="P27" s="189"/>
-      <c r="Q27" s="191"/>
-      <c r="R27" s="192"/>
+      <c r="N27" s="173"/>
+      <c r="O27" s="174"/>
+      <c r="P27" s="174"/>
+      <c r="Q27" s="176"/>
+      <c r="R27" s="177"/>
       <c r="S27" s="11"/>
     </row>
     <row r="28" spans="1:19" ht="15.75">
       <c r="A28" s="1"/>
-      <c r="C28" s="29"/>
+      <c r="C28" s="25"/>
       <c r="D28" s="8"/>
       <c r="E28" s="7"/>
       <c r="G28" s="7"/>
@@ -3535,15 +3547,15 @@
       <c r="I28" s="7"/>
       <c r="J28" s="7"/>
       <c r="K28" s="7"/>
-      <c r="L28" s="61" t="s">
-        <v>38</v>
-      </c>
-      <c r="M28" s="62"/>
-      <c r="N28" s="62"/>
-      <c r="O28" s="63"/>
-      <c r="P28" s="64">
+      <c r="L28" s="186" t="s">
+        <v>37</v>
+      </c>
+      <c r="M28" s="187"/>
+      <c r="N28" s="187"/>
+      <c r="O28" s="51"/>
+      <c r="P28" s="52">
         <f>SUM(P3:P26)</f>
-        <v>365.11730000000006</v>
+        <v>248.20189999999997</v>
       </c>
       <c r="Q28" s="7"/>
       <c r="R28" s="7"/>
@@ -3551,23 +3563,23 @@
     </row>
     <row r="29" spans="1:19" ht="16.5" thickBot="1">
       <c r="A29" s="1"/>
-      <c r="C29" s="29"/>
-      <c r="E29" s="33"/>
-      <c r="F29" s="33"/>
+      <c r="C29" s="25"/>
+      <c r="E29" s="29"/>
+      <c r="F29" s="29"/>
       <c r="G29" s="7"/>
       <c r="H29" s="7"/>
       <c r="I29" s="7"/>
       <c r="J29" s="7"/>
       <c r="K29" s="7"/>
-      <c r="L29" s="65" t="s">
-        <v>39</v>
-      </c>
-      <c r="M29" s="66"/>
-      <c r="N29" s="66"/>
-      <c r="O29" s="58"/>
-      <c r="P29" s="67">
+      <c r="L29" s="188" t="s">
+        <v>38</v>
+      </c>
+      <c r="M29" s="189"/>
+      <c r="N29" s="189"/>
+      <c r="O29" s="48"/>
+      <c r="P29" s="53">
         <f>P28/5</f>
-        <v>73.023460000000014</v>
+        <v>49.640379999999993</v>
       </c>
       <c r="Q29" s="7"/>
       <c r="R29" s="7"/>
@@ -3575,35 +3587,35 @@
     </row>
     <row r="30" spans="1:19" ht="15.75">
       <c r="A30" s="1"/>
-      <c r="C30" s="29"/>
-      <c r="E30" s="33"/>
-      <c r="F30" s="33"/>
+      <c r="C30" s="25"/>
+      <c r="E30" s="29"/>
+      <c r="F30" s="29"/>
       <c r="G30" s="7"/>
       <c r="H30" s="7"/>
       <c r="I30" s="7"/>
       <c r="J30" s="7"/>
       <c r="K30" s="7"/>
-      <c r="L30" s="45"/>
-      <c r="M30" s="54" t="s">
-        <v>165</v>
-      </c>
-      <c r="N30" s="25"/>
-      <c r="O30" s="46"/>
-      <c r="P30" s="60"/>
+      <c r="L30" s="38"/>
+      <c r="M30" s="179" t="s">
+        <v>160</v>
+      </c>
+      <c r="N30" s="180"/>
+      <c r="O30" s="39"/>
+      <c r="P30" s="50"/>
       <c r="Q30" s="7"/>
       <c r="R30" s="7"/>
       <c r="S30" s="11"/>
     </row>
     <row r="31" spans="1:19" ht="15.75">
       <c r="A31" s="1"/>
-      <c r="D31" s="32"/>
-      <c r="E31" s="33"/>
-      <c r="M31" s="54" t="s">
-        <v>44</v>
-      </c>
-      <c r="N31" s="25"/>
+      <c r="D31" s="28"/>
+      <c r="E31" s="29"/>
+      <c r="M31" s="179" t="s">
+        <v>43</v>
+      </c>
+      <c r="N31" s="180"/>
       <c r="O31" s="21"/>
-      <c r="P31" s="55">
+      <c r="P31" s="47">
         <v>213.77</v>
       </c>
       <c r="R31" s="11"/>
@@ -3611,23 +3623,23 @@
     </row>
     <row r="32" spans="1:19" ht="16.5" thickBot="1">
       <c r="A32" s="1"/>
-      <c r="D32" s="33"/>
-      <c r="M32" s="56" t="s">
-        <v>45</v>
-      </c>
-      <c r="N32" s="57"/>
-      <c r="O32" s="58"/>
-      <c r="P32" s="59">
+      <c r="D32" s="29"/>
+      <c r="M32" s="181" t="s">
+        <v>44</v>
+      </c>
+      <c r="N32" s="182"/>
+      <c r="O32" s="48"/>
+      <c r="P32" s="49">
         <f>P31+P28</f>
-        <v>578.8873000000001</v>
+        <v>461.97190000000001</v>
       </c>
       <c r="R32" s="11"/>
       <c r="S32" s="11"/>
     </row>
     <row r="33" spans="1:19">
       <c r="A33" s="1"/>
-      <c r="C33" s="30"/>
-      <c r="D33" s="33"/>
+      <c r="C33" s="26"/>
+      <c r="D33" s="29"/>
       <c r="M33" s="20"/>
       <c r="R33" s="11"/>
       <c r="S33" s="11"/>
@@ -3846,10 +3858,11 @@
     <hyperlink ref="N22" r:id="rId18" xr:uid="{8E22EBA9-5C52-408B-A65B-4F115F1CD0F7}"/>
     <hyperlink ref="N23" r:id="rId19" xr:uid="{0A7E773D-5A3D-486C-84CA-8D29060909A3}"/>
     <hyperlink ref="N25" r:id="rId20" xr:uid="{79B90123-86F4-4C7F-BE0B-E5B7C590F601}"/>
-    <hyperlink ref="N11" r:id="rId21" xr:uid="{D571A1A4-A3B8-476C-81AA-A10E0576C945}"/>
+    <hyperlink ref="N11" r:id="rId21" display="Aliexpress" xr:uid="{D571A1A4-A3B8-476C-81AA-A10E0576C945}"/>
+    <hyperlink ref="N24" r:id="rId22" xr:uid="{552B4167-57FF-43F1-B0A5-FDF3A29237A4}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId22"/>
+  <pageSetup orientation="portrait" r:id="rId23"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>

</xml_diff>

<commit_message>
#50 completed. BOM Revised.
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/eSpark-BOM(5 Boards).xlsx
+++ b/Deliverables/BOM/eSpark-BOM(5 Boards).xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24931"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\Melih-SoundSensor\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7DCCF14-03CB-4DC0-922D-DC993A177CE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="563"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -30,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="175">
   <si>
     <t>S. No.</t>
   </si>
@@ -200,9 +199,6 @@
     <t>CAP CER 1UF 25V X5R 0603</t>
   </si>
   <si>
-    <t>C3, C5, C7, C9, C11, C13, C15, C17, C20, C27, C29, C53, C55, C70, C72</t>
-  </si>
-  <si>
     <t>CC0603KRX5R8BB105</t>
   </si>
   <si>
@@ -299,9 +295,6 @@
     <t>RES SMD 100K OHM 5% 1/5W 0603</t>
   </si>
   <si>
-    <t>R1, R2</t>
-  </si>
-  <si>
     <t>CRGH0603J100K</t>
   </si>
   <si>
@@ -387,9 +380,6 @@
   </si>
   <si>
     <t>2 Pin JST Connector</t>
-  </si>
-  <si>
-    <t>SB1, SB2, SB3, SB8, SB9, SB10, SB11, SB12, SB13, SB14, SB15, SB16, SB17, SB18, SB19, SB20, SB21, SB22, SB23, SB24, SB25, SB26, SB27, SB28, SB29, SB30, SB32, SB34, SB35, SB36, SB37, SB38, SB40, SB41, SB42, SB44, SB45, SB46, SB47, SB48, SB49, SB50</t>
   </si>
   <si>
     <t xml:space="preserve">Connector </t>
@@ -546,12 +536,33 @@
   </si>
   <si>
     <t>Amphenol ICC</t>
+  </si>
+  <si>
+    <t>C3, C5, C7, C9, C11, C13, C15, C17, C20, C27, C29, C53, C55, C70, C72,C#1, C#2</t>
+  </si>
+  <si>
+    <t>R1, R2, R3</t>
+  </si>
+  <si>
+    <t>SB1, SB2, SB3, SB4, SB5, SB8, SB9, SB10, SB11, SB12, SB13, SB14, SB15, SB16, SB17, SB18, SB19, SB20, SB21, SB22, SB23, SB24, SB25, SB26, SB27, SB28, SB29, SB30, SB32, SB34, SB35, SB36, SB37, SB38, SB40, SB41, SB42, SB44, SB45, SB46, SB47, SB48, SB49, SB50, SB70, SB71, SB72</t>
+  </si>
+  <si>
+    <t>Aliexpress</t>
+  </si>
+  <si>
+    <t>Alkaline Battery 2500mAh</t>
+  </si>
+  <si>
+    <t>Energizer</t>
+  </si>
+  <si>
+    <t>5V Adaptor</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
@@ -741,8 +752,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <strike/>
+      <u/>
       <sz val="10"/>
+      <color rgb="FF0070C0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -798,7 +810,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="34">
+  <borders count="35">
     <border>
       <left/>
       <right/>
@@ -1097,39 +1109,11 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color auto="1"/>
       </left>
       <right style="thin">
         <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
       </right>
       <top style="medium">
         <color indexed="64"/>
@@ -1245,6 +1229,45 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -1254,7 +1277,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="195">
+  <cellXfs count="200">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1355,7 +1378,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="13" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1368,10 +1391,10 @@
     <xf numFmtId="165" fontId="13" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -1381,7 +1404,7 @@
     <xf numFmtId="0" fontId="14" fillId="7" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="7" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="9" fillId="7" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1394,10 +1417,6 @@
     <xf numFmtId="165" fontId="4" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1467,25 +1486,25 @@
     <xf numFmtId="164" fontId="19" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1620,7 +1639,7 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="9" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="26" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1635,19 +1654,19 @@
     <xf numFmtId="164" fontId="23" fillId="0" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="30" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="28" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="24" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="28" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="23" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="26" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1710,7 +1729,7 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="26" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="7" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1719,9 +1738,6 @@
     <xf numFmtId="0" fontId="22" fillId="7" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="8" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1752,37 +1768,19 @@
     <xf numFmtId="165" fontId="10" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="24" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="4" borderId="24" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1800,12 +1798,6 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1818,12 +1810,58 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="11" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="24" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="31" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="29" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2099,8 +2137,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S45"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:S46"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6.140625" style="2" customWidth="1"/>
@@ -2125,26 +2163,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="16.5" thickBot="1">
-      <c r="A1" s="183" t="s">
-        <v>163</v>
-      </c>
-      <c r="B1" s="184"/>
-      <c r="C1" s="184"/>
-      <c r="D1" s="184"/>
-      <c r="E1" s="184"/>
-      <c r="F1" s="184"/>
-      <c r="G1" s="184"/>
-      <c r="H1" s="184"/>
-      <c r="I1" s="184"/>
-      <c r="J1" s="184"/>
-      <c r="K1" s="184"/>
-      <c r="L1" s="184"/>
-      <c r="M1" s="184"/>
-      <c r="N1" s="184"/>
-      <c r="O1" s="184"/>
-      <c r="P1" s="184"/>
-      <c r="Q1" s="184"/>
-      <c r="R1" s="185"/>
+      <c r="A1" s="174" t="s">
+        <v>160</v>
+      </c>
+      <c r="B1" s="175"/>
+      <c r="C1" s="175"/>
+      <c r="D1" s="175"/>
+      <c r="E1" s="175"/>
+      <c r="F1" s="175"/>
+      <c r="G1" s="175"/>
+      <c r="H1" s="175"/>
+      <c r="I1" s="175"/>
+      <c r="J1" s="175"/>
+      <c r="K1" s="175"/>
+      <c r="L1" s="175"/>
+      <c r="M1" s="175"/>
+      <c r="N1" s="175"/>
+      <c r="O1" s="175"/>
+      <c r="P1" s="175"/>
+      <c r="Q1" s="175"/>
+      <c r="R1" s="176"/>
     </row>
     <row r="2" spans="1:19" ht="16.5" thickBot="1">
       <c r="A2" s="3" t="s">
@@ -2206,50 +2244,50 @@
       <c r="A3" s="6">
         <v>1</v>
       </c>
-      <c r="B3" s="190" t="s">
+      <c r="B3" s="179" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="115" t="s">
+      <c r="C3" s="113" t="s">
         <v>49</v>
       </c>
-      <c r="D3" s="116" t="s">
+      <c r="D3" s="114" t="s">
         <v>50</v>
       </c>
-      <c r="E3" s="117" t="s">
+      <c r="E3" s="115" t="s">
         <v>51</v>
       </c>
-      <c r="F3" s="117" t="s">
+      <c r="F3" s="115" t="s">
         <v>52</v>
       </c>
-      <c r="G3" s="54" t="s">
-        <v>121</v>
-      </c>
-      <c r="H3" s="55" t="s">
-        <v>122</v>
-      </c>
-      <c r="I3" s="56" t="s">
+      <c r="G3" s="52" t="s">
+        <v>118</v>
+      </c>
+      <c r="H3" s="53" t="s">
+        <v>119</v>
+      </c>
+      <c r="I3" s="54" t="s">
         <v>39</v>
       </c>
-      <c r="J3" s="116" t="s">
+      <c r="J3" s="114" t="s">
         <v>20</v>
       </c>
-      <c r="K3" s="57">
+      <c r="K3" s="55">
         <v>20</v>
       </c>
-      <c r="L3" s="118">
+      <c r="L3" s="116">
         <v>3</v>
       </c>
-      <c r="M3" s="58">
+      <c r="M3" s="56">
         <f>L3*5</f>
         <v>15</v>
       </c>
-      <c r="N3" s="119" t="s">
+      <c r="N3" s="117" t="s">
         <v>16</v>
       </c>
-      <c r="O3" s="59">
+      <c r="O3" s="57">
         <v>2.58E-2</v>
       </c>
-      <c r="P3" s="60">
+      <c r="P3" s="58">
         <f>O3*K3</f>
         <v>0.51600000000000001</v>
       </c>
@@ -2260,49 +2298,49 @@
       <c r="A4" s="6">
         <v>2</v>
       </c>
-      <c r="B4" s="191"/>
-      <c r="C4" s="120" t="s">
+      <c r="B4" s="180"/>
+      <c r="C4" s="118" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="121" t="s">
+      <c r="D4" s="119" t="s">
         <v>53</v>
       </c>
-      <c r="E4" s="122" t="s">
+      <c r="E4" s="120" t="s">
         <v>51</v>
       </c>
-      <c r="F4" s="122" t="s">
+      <c r="F4" s="120" t="s">
         <v>54</v>
       </c>
-      <c r="G4" s="61" t="s">
-        <v>121</v>
-      </c>
-      <c r="H4" s="62" t="s">
-        <v>123</v>
-      </c>
-      <c r="I4" s="63" t="s">
+      <c r="G4" s="59" t="s">
+        <v>118</v>
+      </c>
+      <c r="H4" s="60" t="s">
+        <v>120</v>
+      </c>
+      <c r="I4" s="61" t="s">
         <v>39</v>
       </c>
-      <c r="J4" s="121" t="s">
-        <v>72</v>
-      </c>
-      <c r="K4" s="64">
+      <c r="J4" s="119" t="s">
+        <v>71</v>
+      </c>
+      <c r="K4" s="62">
         <v>20</v>
       </c>
-      <c r="L4" s="123">
+      <c r="L4" s="121">
         <v>1</v>
       </c>
-      <c r="M4" s="65">
-        <f t="shared" ref="M4:M27" si="0">L4*5</f>
+      <c r="M4" s="63">
+        <f t="shared" ref="M4:M28" si="0">L4*5</f>
         <v>5</v>
       </c>
-      <c r="N4" s="124" t="s">
+      <c r="N4" s="122" t="s">
         <v>16</v>
       </c>
-      <c r="O4" s="66">
+      <c r="O4" s="64">
         <v>2.0299999999999999E-2</v>
       </c>
-      <c r="P4" s="67">
-        <f t="shared" ref="P4:P25" si="1">O4*K4</f>
+      <c r="P4" s="65">
+        <f t="shared" ref="P4:P28" si="1">O4*K4</f>
         <v>0.40599999999999997</v>
       </c>
       <c r="Q4" s="14"/>
@@ -2312,48 +2350,48 @@
       <c r="A5" s="6">
         <v>3</v>
       </c>
-      <c r="B5" s="191"/>
-      <c r="C5" s="120" t="s">
+      <c r="B5" s="180"/>
+      <c r="C5" s="118" t="s">
         <v>55</v>
       </c>
-      <c r="D5" s="125" t="s">
+      <c r="D5" s="123" t="s">
+        <v>168</v>
+      </c>
+      <c r="E5" s="119" t="s">
+        <v>51</v>
+      </c>
+      <c r="F5" s="119" t="s">
         <v>56</v>
       </c>
-      <c r="E5" s="121" t="s">
-        <v>51</v>
-      </c>
-      <c r="F5" s="121" t="s">
-        <v>57</v>
-      </c>
-      <c r="G5" s="68" t="s">
-        <v>124</v>
-      </c>
-      <c r="H5" s="62" t="s">
-        <v>125</v>
-      </c>
-      <c r="I5" s="63" t="s">
+      <c r="G5" s="66" t="s">
+        <v>121</v>
+      </c>
+      <c r="H5" s="60" t="s">
+        <v>122</v>
+      </c>
+      <c r="I5" s="61" t="s">
         <v>39</v>
       </c>
-      <c r="J5" s="121" t="s">
+      <c r="J5" s="119" t="s">
         <v>15</v>
       </c>
-      <c r="K5" s="64">
+      <c r="K5" s="62">
         <v>100</v>
       </c>
-      <c r="L5" s="123">
-        <v>15</v>
-      </c>
-      <c r="M5" s="65">
+      <c r="L5" s="121">
+        <v>17</v>
+      </c>
+      <c r="M5" s="63">
         <f t="shared" si="0"/>
-        <v>75</v>
-      </c>
-      <c r="N5" s="124" t="s">
+        <v>85</v>
+      </c>
+      <c r="N5" s="122" t="s">
         <v>16</v>
       </c>
-      <c r="O5" s="66">
+      <c r="O5" s="64">
         <v>7.3000000000000001E-3</v>
       </c>
-      <c r="P5" s="67">
+      <c r="P5" s="65">
         <f t="shared" si="1"/>
         <v>0.73</v>
       </c>
@@ -2365,48 +2403,48 @@
       <c r="A6" s="6">
         <v>4</v>
       </c>
-      <c r="B6" s="191"/>
-      <c r="C6" s="120" t="s">
+      <c r="B6" s="180"/>
+      <c r="C6" s="118" t="s">
+        <v>57</v>
+      </c>
+      <c r="D6" s="119" t="s">
         <v>58</v>
       </c>
-      <c r="D6" s="121" t="s">
+      <c r="E6" s="120" t="s">
         <v>59</v>
       </c>
-      <c r="E6" s="122" t="s">
+      <c r="F6" s="120" t="s">
         <v>60</v>
       </c>
-      <c r="F6" s="122" t="s">
-        <v>61</v>
-      </c>
-      <c r="G6" s="68" t="s">
-        <v>124</v>
-      </c>
-      <c r="H6" s="62" t="s">
-        <v>126</v>
-      </c>
-      <c r="I6" s="63" t="s">
+      <c r="G6" s="66" t="s">
+        <v>121</v>
+      </c>
+      <c r="H6" s="60" t="s">
+        <v>123</v>
+      </c>
+      <c r="I6" s="61" t="s">
         <v>39</v>
       </c>
-      <c r="J6" s="121" t="s">
-        <v>73</v>
-      </c>
-      <c r="K6" s="64">
+      <c r="J6" s="119" t="s">
+        <v>72</v>
+      </c>
+      <c r="K6" s="62">
         <v>100</v>
       </c>
-      <c r="L6" s="123">
+      <c r="L6" s="121">
         <v>8</v>
       </c>
-      <c r="M6" s="65">
+      <c r="M6" s="63">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="N6" s="126" t="s">
+      <c r="N6" s="124" t="s">
         <v>16</v>
       </c>
-      <c r="O6" s="66">
+      <c r="O6" s="64">
         <v>3.7000000000000002E-3</v>
       </c>
-      <c r="P6" s="67">
+      <c r="P6" s="65">
         <f t="shared" si="1"/>
         <v>0.37</v>
       </c>
@@ -2418,48 +2456,48 @@
       <c r="A7" s="6">
         <v>5</v>
       </c>
-      <c r="B7" s="191"/>
-      <c r="C7" s="120" t="s">
+      <c r="B7" s="180"/>
+      <c r="C7" s="118" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="125" t="s">
-        <v>62</v>
-      </c>
-      <c r="E7" s="121" t="s">
+      <c r="D7" s="123" t="s">
+        <v>61</v>
+      </c>
+      <c r="E7" s="119" t="s">
         <v>51</v>
       </c>
-      <c r="F7" s="121" t="s">
+      <c r="F7" s="119" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="68" t="s">
+      <c r="G7" s="66" t="s">
+        <v>121</v>
+      </c>
+      <c r="H7" s="60" t="s">
         <v>124</v>
       </c>
-      <c r="H7" s="62" t="s">
-        <v>127</v>
-      </c>
-      <c r="I7" s="63" t="s">
+      <c r="I7" s="61" t="s">
         <v>39</v>
       </c>
-      <c r="J7" s="121" t="s">
+      <c r="J7" s="119" t="s">
         <v>19</v>
       </c>
-      <c r="K7" s="64">
+      <c r="K7" s="62">
         <v>150</v>
       </c>
-      <c r="L7" s="123">
+      <c r="L7" s="121">
         <v>24</v>
       </c>
-      <c r="M7" s="65">
+      <c r="M7" s="63">
         <f t="shared" si="0"/>
         <v>120</v>
       </c>
-      <c r="N7" s="126" t="s">
+      <c r="N7" s="124" t="s">
         <v>16</v>
       </c>
-      <c r="O7" s="66">
+      <c r="O7" s="64">
         <v>7.9000000000000008E-3</v>
       </c>
-      <c r="P7" s="67">
+      <c r="P7" s="65">
         <f t="shared" si="1"/>
         <v>1.1850000000000001</v>
       </c>
@@ -2471,48 +2509,48 @@
       <c r="A8" s="6">
         <v>6</v>
       </c>
-      <c r="B8" s="191"/>
-      <c r="C8" s="120" t="s">
+      <c r="B8" s="180"/>
+      <c r="C8" s="118" t="s">
+        <v>62</v>
+      </c>
+      <c r="D8" s="119" t="s">
         <v>63</v>
       </c>
-      <c r="D8" s="121" t="s">
+      <c r="E8" s="120" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" s="120" t="s">
         <v>64</v>
       </c>
-      <c r="E8" s="122" t="s">
-        <v>51</v>
-      </c>
-      <c r="F8" s="122" t="s">
-        <v>65</v>
-      </c>
-      <c r="G8" s="68" t="s">
-        <v>128</v>
-      </c>
-      <c r="H8" s="69" t="s">
-        <v>129</v>
-      </c>
-      <c r="I8" s="63" t="s">
+      <c r="G8" s="66" t="s">
+        <v>125</v>
+      </c>
+      <c r="H8" s="67" t="s">
+        <v>126</v>
+      </c>
+      <c r="I8" s="61" t="s">
         <v>39</v>
       </c>
-      <c r="J8" s="121" t="s">
-        <v>74</v>
-      </c>
-      <c r="K8" s="68">
+      <c r="J8" s="119" t="s">
+        <v>73</v>
+      </c>
+      <c r="K8" s="66">
         <v>10</v>
       </c>
-      <c r="L8" s="123">
+      <c r="L8" s="121">
         <v>1</v>
       </c>
-      <c r="M8" s="65">
+      <c r="M8" s="63">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N8" s="126" t="s">
+      <c r="N8" s="124" t="s">
         <v>16</v>
       </c>
-      <c r="O8" s="66">
+      <c r="O8" s="64">
         <v>4.4299999999999999E-2</v>
       </c>
-      <c r="P8" s="67">
+      <c r="P8" s="65">
         <f t="shared" si="1"/>
         <v>0.443</v>
       </c>
@@ -2524,48 +2562,48 @@
       <c r="A9" s="6">
         <v>7</v>
       </c>
-      <c r="B9" s="191"/>
-      <c r="C9" s="120" t="s">
+      <c r="B9" s="180"/>
+      <c r="C9" s="118" t="s">
+        <v>65</v>
+      </c>
+      <c r="D9" s="119" t="s">
         <v>66</v>
       </c>
-      <c r="D9" s="121" t="s">
+      <c r="E9" s="120" t="s">
+        <v>51</v>
+      </c>
+      <c r="F9" s="120" t="s">
         <v>67</v>
       </c>
-      <c r="E9" s="122" t="s">
-        <v>51</v>
-      </c>
-      <c r="F9" s="122" t="s">
-        <v>68</v>
-      </c>
-      <c r="G9" s="68" t="s">
-        <v>124</v>
-      </c>
-      <c r="H9" s="62" t="s">
-        <v>130</v>
-      </c>
-      <c r="I9" s="63" t="s">
+      <c r="G9" s="66" t="s">
+        <v>121</v>
+      </c>
+      <c r="H9" s="60" t="s">
+        <v>127</v>
+      </c>
+      <c r="I9" s="61" t="s">
         <v>39</v>
       </c>
-      <c r="J9" s="121" t="s">
-        <v>75</v>
-      </c>
-      <c r="K9" s="68">
+      <c r="J9" s="119" t="s">
+        <v>74</v>
+      </c>
+      <c r="K9" s="66">
         <v>100</v>
       </c>
-      <c r="L9" s="123">
+      <c r="L9" s="121">
         <v>6</v>
       </c>
-      <c r="M9" s="65">
+      <c r="M9" s="63">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="N9" s="124" t="s">
+      <c r="N9" s="122" t="s">
         <v>16</v>
       </c>
-      <c r="O9" s="66">
+      <c r="O9" s="64">
         <v>3.2000000000000002E-3</v>
       </c>
-      <c r="P9" s="67">
+      <c r="P9" s="65">
         <f t="shared" si="1"/>
         <v>0.32</v>
       </c>
@@ -2577,48 +2615,48 @@
       <c r="A10" s="6">
         <v>8</v>
       </c>
-      <c r="B10" s="192"/>
-      <c r="C10" s="127" t="s">
+      <c r="B10" s="181"/>
+      <c r="C10" s="125" t="s">
+        <v>68</v>
+      </c>
+      <c r="D10" s="126" t="s">
         <v>69</v>
       </c>
-      <c r="D10" s="128" t="s">
+      <c r="E10" s="127" t="s">
+        <v>51</v>
+      </c>
+      <c r="F10" s="127" t="s">
         <v>70</v>
       </c>
-      <c r="E10" s="129" t="s">
-        <v>51</v>
-      </c>
-      <c r="F10" s="129" t="s">
-        <v>71</v>
-      </c>
-      <c r="G10" s="70" t="s">
-        <v>124</v>
-      </c>
-      <c r="H10" s="71" t="s">
-        <v>131</v>
-      </c>
-      <c r="I10" s="72" t="s">
+      <c r="G10" s="68" t="s">
+        <v>121</v>
+      </c>
+      <c r="H10" s="69" t="s">
+        <v>128</v>
+      </c>
+      <c r="I10" s="70" t="s">
         <v>39</v>
       </c>
-      <c r="J10" s="129" t="s">
-        <v>76</v>
-      </c>
-      <c r="K10" s="70">
+      <c r="J10" s="127" t="s">
+        <v>75</v>
+      </c>
+      <c r="K10" s="68">
         <v>100</v>
       </c>
-      <c r="L10" s="130">
+      <c r="L10" s="128">
         <v>16</v>
       </c>
-      <c r="M10" s="73">
+      <c r="M10" s="71">
         <f t="shared" si="0"/>
         <v>80</v>
       </c>
-      <c r="N10" s="131" t="s">
+      <c r="N10" s="129" t="s">
         <v>16</v>
       </c>
-      <c r="O10" s="74">
+      <c r="O10" s="72">
         <v>1.7299999999999999E-2</v>
       </c>
-      <c r="P10" s="75">
+      <c r="P10" s="73">
         <f t="shared" si="1"/>
         <v>1.73</v>
       </c>
@@ -2631,54 +2669,54 @@
         <v>9</v>
       </c>
       <c r="B11" s="33" t="s">
-        <v>80</v>
-      </c>
-      <c r="C11" s="132" t="s">
+        <v>79</v>
+      </c>
+      <c r="C11" s="130" t="s">
+        <v>76</v>
+      </c>
+      <c r="D11" s="131" t="s">
         <v>77</v>
       </c>
-      <c r="D11" s="133" t="s">
+      <c r="E11" s="132" t="s">
+        <v>28</v>
+      </c>
+      <c r="F11" s="132" t="s">
         <v>78</v>
       </c>
-      <c r="E11" s="134" t="s">
-        <v>28</v>
-      </c>
-      <c r="F11" s="134" t="s">
-        <v>79</v>
-      </c>
-      <c r="G11" s="76" t="s">
-        <v>159</v>
-      </c>
-      <c r="H11" s="77" t="s">
-        <v>157</v>
-      </c>
-      <c r="I11" s="78" t="s">
-        <v>158</v>
-      </c>
-      <c r="J11" s="79" t="s">
+      <c r="G11" s="74" t="s">
+        <v>156</v>
+      </c>
+      <c r="H11" s="75" t="s">
+        <v>154</v>
+      </c>
+      <c r="I11" s="76" t="s">
+        <v>155</v>
+      </c>
+      <c r="J11" s="77" t="s">
         <v>22</v>
       </c>
-      <c r="K11" s="79">
+      <c r="K11" s="77">
         <v>42</v>
       </c>
-      <c r="L11" s="80">
+      <c r="L11" s="78">
         <v>8</v>
       </c>
-      <c r="M11" s="80">
+      <c r="M11" s="78">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="N11" s="135" t="s">
-        <v>166</v>
-      </c>
-      <c r="O11" s="81">
+      <c r="N11" s="133" t="s">
+        <v>163</v>
+      </c>
+      <c r="O11" s="79">
         <v>3.68</v>
       </c>
-      <c r="P11" s="82">
+      <c r="P11" s="80">
         <f t="shared" si="1"/>
         <v>154.56</v>
       </c>
       <c r="Q11" s="42" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="R11" s="43"/>
       <c r="S11" s="11"/>
@@ -2690,47 +2728,47 @@
       <c r="B12" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="136" t="s">
+      <c r="C12" s="134" t="s">
+        <v>80</v>
+      </c>
+      <c r="D12" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="136" t="s">
+        <v>28</v>
+      </c>
+      <c r="F12" s="136" t="s">
         <v>81</v>
       </c>
-      <c r="D12" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="138" t="s">
-        <v>28</v>
-      </c>
-      <c r="F12" s="138" t="s">
-        <v>82</v>
-      </c>
-      <c r="G12" s="83" t="s">
-        <v>132</v>
-      </c>
-      <c r="H12" s="84" t="s">
-        <v>133</v>
-      </c>
-      <c r="I12" s="85" t="s">
+      <c r="G12" s="81" t="s">
+        <v>129</v>
+      </c>
+      <c r="H12" s="82" t="s">
+        <v>130</v>
+      </c>
+      <c r="I12" s="83" t="s">
         <v>39</v>
       </c>
-      <c r="J12" s="86" t="s">
+      <c r="J12" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="K12" s="86">
+      <c r="K12" s="84">
         <v>10</v>
       </c>
-      <c r="L12" s="87">
+      <c r="L12" s="85">
         <v>1</v>
       </c>
-      <c r="M12" s="87">
+      <c r="M12" s="85">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N12" s="139" t="s">
+      <c r="N12" s="137" t="s">
         <v>16</v>
       </c>
-      <c r="O12" s="88">
+      <c r="O12" s="86">
         <v>6.0600000000000001E-2</v>
       </c>
-      <c r="P12" s="89">
+      <c r="P12" s="87">
         <f t="shared" si="1"/>
         <v>0.60599999999999998</v>
       </c>
@@ -2742,50 +2780,50 @@
       <c r="A13" s="6">
         <v>11</v>
       </c>
-      <c r="B13" s="190" t="s">
+      <c r="B13" s="179" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="140" t="s">
+      <c r="C13" s="138" t="s">
+        <v>82</v>
+      </c>
+      <c r="D13" s="139" t="s">
+        <v>33</v>
+      </c>
+      <c r="E13" s="139" t="s">
+        <v>28</v>
+      </c>
+      <c r="F13" s="139" t="s">
         <v>83</v>
       </c>
-      <c r="D13" s="141" t="s">
-        <v>33</v>
-      </c>
-      <c r="E13" s="141" t="s">
-        <v>28</v>
-      </c>
-      <c r="F13" s="141" t="s">
-        <v>84</v>
-      </c>
-      <c r="G13" s="90" t="s">
-        <v>134</v>
-      </c>
-      <c r="H13" s="91" t="s">
-        <v>135</v>
-      </c>
-      <c r="I13" s="92" t="s">
+      <c r="G13" s="88" t="s">
+        <v>131</v>
+      </c>
+      <c r="H13" s="89" t="s">
+        <v>132</v>
+      </c>
+      <c r="I13" s="90" t="s">
         <v>39</v>
       </c>
-      <c r="J13" s="93" t="s">
+      <c r="J13" s="91" t="s">
         <v>22</v>
       </c>
-      <c r="K13" s="93">
+      <c r="K13" s="91">
         <v>7</v>
       </c>
-      <c r="L13" s="94">
+      <c r="L13" s="92">
         <v>1</v>
       </c>
-      <c r="M13" s="94">
+      <c r="M13" s="92">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N13" s="142" t="s">
+      <c r="N13" s="140" t="s">
         <v>16</v>
       </c>
-      <c r="O13" s="95">
+      <c r="O13" s="93">
         <v>0.25650000000000001</v>
       </c>
-      <c r="P13" s="96">
+      <c r="P13" s="94">
         <f>O13*K13</f>
         <v>1.7955000000000001</v>
       </c>
@@ -2797,48 +2835,48 @@
       <c r="A14" s="6">
         <v>12</v>
       </c>
-      <c r="B14" s="192"/>
-      <c r="C14" s="143" t="s">
+      <c r="B14" s="181"/>
+      <c r="C14" s="141" t="s">
+        <v>84</v>
+      </c>
+      <c r="D14" s="142" t="s">
         <v>85</v>
       </c>
-      <c r="D14" s="144" t="s">
+      <c r="E14" s="143" t="s">
+        <v>28</v>
+      </c>
+      <c r="F14" s="143" t="s">
         <v>86</v>
       </c>
-      <c r="E14" s="145" t="s">
-        <v>28</v>
-      </c>
-      <c r="F14" s="145" t="s">
-        <v>87</v>
-      </c>
-      <c r="G14" s="97" t="s">
-        <v>136</v>
-      </c>
-      <c r="H14" s="98" t="s">
-        <v>137</v>
-      </c>
-      <c r="I14" s="99" t="s">
+      <c r="G14" s="95" t="s">
+        <v>133</v>
+      </c>
+      <c r="H14" s="96" t="s">
+        <v>134</v>
+      </c>
+      <c r="I14" s="97" t="s">
         <v>39</v>
       </c>
-      <c r="J14" s="100" t="s">
+      <c r="J14" s="98" t="s">
         <v>22</v>
       </c>
-      <c r="K14" s="100">
+      <c r="K14" s="98">
         <v>7</v>
       </c>
-      <c r="L14" s="101">
+      <c r="L14" s="99">
         <v>2</v>
       </c>
-      <c r="M14" s="87">
+      <c r="M14" s="85">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="N14" s="146" t="s">
+      <c r="N14" s="144" t="s">
         <v>16</v>
       </c>
-      <c r="O14" s="102">
+      <c r="O14" s="100">
         <v>0.1215</v>
       </c>
-      <c r="P14" s="89">
+      <c r="P14" s="87">
         <f t="shared" si="1"/>
         <v>0.85050000000000003</v>
       </c>
@@ -2850,50 +2888,50 @@
       <c r="A15" s="6">
         <v>13</v>
       </c>
-      <c r="B15" s="190" t="s">
+      <c r="B15" s="179" t="s">
         <v>23</v>
       </c>
-      <c r="C15" s="140" t="s">
+      <c r="C15" s="138" t="s">
+        <v>87</v>
+      </c>
+      <c r="D15" s="139" t="s">
+        <v>169</v>
+      </c>
+      <c r="E15" s="114" t="s">
+        <v>24</v>
+      </c>
+      <c r="F15" s="145" t="s">
         <v>88</v>
       </c>
-      <c r="D15" s="141" t="s">
-        <v>89</v>
-      </c>
-      <c r="E15" s="116" t="s">
-        <v>24</v>
-      </c>
-      <c r="F15" s="147" t="s">
-        <v>90</v>
-      </c>
-      <c r="G15" s="54" t="s">
-        <v>140</v>
-      </c>
-      <c r="H15" s="55" t="s">
-        <v>139</v>
-      </c>
-      <c r="I15" s="103" t="s">
-        <v>138</v>
-      </c>
-      <c r="J15" s="116" t="s">
-        <v>94</v>
-      </c>
-      <c r="K15" s="104">
+      <c r="G15" s="52" t="s">
+        <v>137</v>
+      </c>
+      <c r="H15" s="53" t="s">
+        <v>136</v>
+      </c>
+      <c r="I15" s="101" t="s">
+        <v>135</v>
+      </c>
+      <c r="J15" s="114" t="s">
+        <v>92</v>
+      </c>
+      <c r="K15" s="102">
         <v>100</v>
       </c>
-      <c r="L15" s="104">
-        <v>2</v>
-      </c>
-      <c r="M15" s="58">
+      <c r="L15" s="102">
+        <v>3</v>
+      </c>
+      <c r="M15" s="56">
         <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="N15" s="148" t="s">
+        <v>15</v>
+      </c>
+      <c r="N15" s="146" t="s">
         <v>16</v>
       </c>
-      <c r="O15" s="59">
+      <c r="O15" s="57">
         <v>1E-3</v>
       </c>
-      <c r="P15" s="60">
+      <c r="P15" s="58">
         <f t="shared" si="1"/>
         <v>0.1</v>
       </c>
@@ -2905,48 +2943,48 @@
       <c r="A16" s="6">
         <v>14</v>
       </c>
-      <c r="B16" s="192"/>
-      <c r="C16" s="143" t="s">
+      <c r="B16" s="181"/>
+      <c r="C16" s="141" t="s">
+        <v>89</v>
+      </c>
+      <c r="D16" s="142" t="s">
+        <v>90</v>
+      </c>
+      <c r="E16" s="143" t="s">
+        <v>24</v>
+      </c>
+      <c r="F16" s="143" t="s">
         <v>91</v>
       </c>
-      <c r="D16" s="144" t="s">
-        <v>92</v>
-      </c>
-      <c r="E16" s="145" t="s">
-        <v>24</v>
-      </c>
-      <c r="F16" s="145" t="s">
-        <v>93</v>
-      </c>
-      <c r="G16" s="97" t="s">
-        <v>124</v>
-      </c>
-      <c r="H16" s="98" t="s">
-        <v>141</v>
-      </c>
-      <c r="I16" s="99" t="s">
+      <c r="G16" s="95" t="s">
+        <v>121</v>
+      </c>
+      <c r="H16" s="96" t="s">
+        <v>138</v>
+      </c>
+      <c r="I16" s="97" t="s">
         <v>39</v>
       </c>
-      <c r="J16" s="145" t="s">
+      <c r="J16" s="143" t="s">
         <v>25</v>
       </c>
-      <c r="K16" s="105">
+      <c r="K16" s="103">
         <v>100</v>
       </c>
-      <c r="L16" s="105">
+      <c r="L16" s="103">
         <v>1</v>
       </c>
-      <c r="M16" s="87">
+      <c r="M16" s="85">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N16" s="149" t="s">
+      <c r="N16" s="147" t="s">
         <v>16</v>
       </c>
-      <c r="O16" s="102">
+      <c r="O16" s="100">
         <v>1.4E-3</v>
       </c>
-      <c r="P16" s="89">
+      <c r="P16" s="87">
         <f t="shared" si="1"/>
         <v>0.13999999999999999</v>
       </c>
@@ -2958,50 +2996,50 @@
       <c r="A17" s="6">
         <v>15</v>
       </c>
-      <c r="B17" s="190" t="s">
-        <v>114</v>
-      </c>
-      <c r="C17" s="140" t="s">
+      <c r="B17" s="179" t="s">
+        <v>112</v>
+      </c>
+      <c r="C17" s="138" t="s">
+        <v>93</v>
+      </c>
+      <c r="D17" s="139" t="s">
+        <v>94</v>
+      </c>
+      <c r="E17" s="114" t="s">
         <v>95</v>
       </c>
-      <c r="D17" s="141" t="s">
+      <c r="F17" s="114" t="s">
         <v>96</v>
       </c>
-      <c r="E17" s="116" t="s">
-        <v>97</v>
-      </c>
-      <c r="F17" s="116" t="s">
-        <v>98</v>
-      </c>
-      <c r="G17" s="54" t="s">
+      <c r="G17" s="52" t="s">
         <v>31</v>
       </c>
-      <c r="H17" s="55" t="s">
-        <v>142</v>
-      </c>
-      <c r="I17" s="56" t="s">
+      <c r="H17" s="53" t="s">
+        <v>139</v>
+      </c>
+      <c r="I17" s="54" t="s">
         <v>39</v>
       </c>
-      <c r="J17" s="57" t="s">
+      <c r="J17" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="K17" s="57">
+      <c r="K17" s="55">
         <v>11</v>
       </c>
-      <c r="L17" s="118">
+      <c r="L17" s="116">
         <v>2</v>
       </c>
-      <c r="M17" s="58">
+      <c r="M17" s="56">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="N17" s="150" t="s">
+      <c r="N17" s="148" t="s">
         <v>16</v>
       </c>
-      <c r="O17" s="59">
+      <c r="O17" s="57">
         <v>0.44729999999999998</v>
       </c>
-      <c r="P17" s="60">
+      <c r="P17" s="58">
         <f t="shared" si="1"/>
         <v>4.9203000000000001</v>
       </c>
@@ -3013,48 +3051,48 @@
       <c r="A18" s="6">
         <v>16</v>
       </c>
-      <c r="B18" s="191"/>
-      <c r="C18" s="151" t="s">
+      <c r="B18" s="180"/>
+      <c r="C18" s="149" t="s">
+        <v>97</v>
+      </c>
+      <c r="D18" s="123" t="s">
+        <v>30</v>
+      </c>
+      <c r="E18" s="119" t="s">
+        <v>98</v>
+      </c>
+      <c r="F18" s="119" t="s">
         <v>99</v>
       </c>
-      <c r="D18" s="125" t="s">
-        <v>30</v>
-      </c>
-      <c r="E18" s="121" t="s">
-        <v>100</v>
-      </c>
-      <c r="F18" s="121" t="s">
-        <v>101</v>
-      </c>
-      <c r="G18" s="63" t="s">
-        <v>143</v>
-      </c>
-      <c r="H18" s="63" t="s">
-        <v>144</v>
-      </c>
-      <c r="I18" s="63" t="s">
+      <c r="G18" s="61" t="s">
+        <v>140</v>
+      </c>
+      <c r="H18" s="61" t="s">
+        <v>141</v>
+      </c>
+      <c r="I18" s="61" t="s">
         <v>39</v>
       </c>
-      <c r="J18" s="64" t="s">
+      <c r="J18" s="62" t="s">
         <v>22</v>
       </c>
-      <c r="K18" s="63">
+      <c r="K18" s="61">
         <v>6</v>
       </c>
-      <c r="L18" s="123">
+      <c r="L18" s="121">
         <v>1</v>
       </c>
-      <c r="M18" s="65">
+      <c r="M18" s="63">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N18" s="126" t="s">
+      <c r="N18" s="124" t="s">
         <v>16</v>
       </c>
-      <c r="O18" s="66">
+      <c r="O18" s="64">
         <v>0.53200000000000003</v>
       </c>
-      <c r="P18" s="67">
+      <c r="P18" s="65">
         <f t="shared" si="1"/>
         <v>3.1920000000000002</v>
       </c>
@@ -3066,53 +3104,53 @@
       <c r="A19" s="6">
         <v>17</v>
       </c>
-      <c r="B19" s="191"/>
-      <c r="C19" s="151" t="s">
+      <c r="B19" s="180"/>
+      <c r="C19" s="149" t="s">
+        <v>100</v>
+      </c>
+      <c r="D19" s="123" t="s">
+        <v>29</v>
+      </c>
+      <c r="E19" s="119" t="s">
+        <v>101</v>
+      </c>
+      <c r="F19" s="119" t="s">
         <v>102</v>
       </c>
-      <c r="D19" s="125" t="s">
-        <v>29</v>
-      </c>
-      <c r="E19" s="121" t="s">
-        <v>103</v>
-      </c>
-      <c r="F19" s="121" t="s">
-        <v>104</v>
-      </c>
-      <c r="G19" s="68" t="s">
+      <c r="G19" s="66" t="s">
         <v>31</v>
       </c>
-      <c r="H19" s="68" t="s">
+      <c r="H19" s="66" t="s">
         <v>22</v>
       </c>
-      <c r="I19" s="64" t="s">
+      <c r="I19" s="62" t="s">
         <v>39</v>
       </c>
-      <c r="J19" s="64" t="s">
+      <c r="J19" s="62" t="s">
         <v>22</v>
       </c>
-      <c r="K19" s="68">
+      <c r="K19" s="66">
         <v>6</v>
       </c>
-      <c r="L19" s="123">
+      <c r="L19" s="121">
         <v>1</v>
       </c>
-      <c r="M19" s="65">
+      <c r="M19" s="63">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N19" s="152" t="s">
-        <v>145</v>
-      </c>
-      <c r="O19" s="106">
+      <c r="N19" s="150" t="s">
+        <v>142</v>
+      </c>
+      <c r="O19" s="104">
         <v>8</v>
       </c>
-      <c r="P19" s="67">
+      <c r="P19" s="65">
         <f t="shared" si="1"/>
         <v>48</v>
       </c>
       <c r="Q19" s="40" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="R19" s="37"/>
       <c r="S19" s="11"/>
@@ -3121,99 +3159,99 @@
       <c r="A20" s="6">
         <v>18</v>
       </c>
-      <c r="B20" s="191"/>
-      <c r="C20" s="161" t="s">
+      <c r="B20" s="180"/>
+      <c r="C20" s="158" t="s">
+        <v>103</v>
+      </c>
+      <c r="D20" s="159" t="s">
+        <v>104</v>
+      </c>
+      <c r="E20" s="160" t="s">
+        <v>144</v>
+      </c>
+      <c r="F20" s="160" t="s">
         <v>105</v>
       </c>
-      <c r="D20" s="162" t="s">
-        <v>106</v>
-      </c>
-      <c r="E20" s="163" t="s">
-        <v>147</v>
-      </c>
-      <c r="F20" s="163" t="s">
-        <v>107</v>
-      </c>
-      <c r="G20" s="164" t="s">
+      <c r="G20" s="161" t="s">
         <v>31</v>
       </c>
-      <c r="H20" s="164" t="s">
+      <c r="H20" s="161" t="s">
         <v>22</v>
       </c>
-      <c r="I20" s="163" t="s">
+      <c r="I20" s="160" t="s">
         <v>39</v>
       </c>
-      <c r="J20" s="163" t="s">
+      <c r="J20" s="160" t="s">
         <v>22</v>
       </c>
-      <c r="K20" s="164"/>
-      <c r="L20" s="165">
+      <c r="K20" s="161"/>
+      <c r="L20" s="162">
         <v>2</v>
       </c>
-      <c r="M20" s="166">
+      <c r="M20" s="163">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="N20" s="167" t="s">
-        <v>166</v>
-      </c>
-      <c r="O20" s="193">
+      <c r="N20" s="164" t="s">
+        <v>163</v>
+      </c>
+      <c r="O20" s="168">
         <v>10.18</v>
       </c>
-      <c r="P20" s="168">
+      <c r="P20" s="165">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="Q20" s="169"/>
-      <c r="R20" s="170"/>
+      <c r="Q20" s="166"/>
+      <c r="R20" s="167"/>
       <c r="S20" s="11"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1">
       <c r="A21" s="6">
         <v>19</v>
       </c>
-      <c r="B21" s="191"/>
-      <c r="C21" s="151" t="s">
+      <c r="B21" s="180"/>
+      <c r="C21" s="149" t="s">
+        <v>106</v>
+      </c>
+      <c r="D21" s="123" t="s">
+        <v>107</v>
+      </c>
+      <c r="E21" s="119" t="s">
+        <v>28</v>
+      </c>
+      <c r="F21" s="119" t="s">
         <v>108</v>
       </c>
-      <c r="D21" s="125" t="s">
-        <v>109</v>
-      </c>
-      <c r="E21" s="121" t="s">
-        <v>28</v>
-      </c>
-      <c r="F21" s="121" t="s">
-        <v>110</v>
-      </c>
-      <c r="G21" s="68" t="s">
-        <v>148</v>
-      </c>
-      <c r="H21" s="68" t="s">
-        <v>149</v>
-      </c>
-      <c r="I21" s="64" t="s">
+      <c r="G21" s="66" t="s">
+        <v>145</v>
+      </c>
+      <c r="H21" s="66" t="s">
+        <v>146</v>
+      </c>
+      <c r="I21" s="62" t="s">
         <v>39</v>
       </c>
-      <c r="J21" s="64" t="s">
+      <c r="J21" s="62" t="s">
         <v>22</v>
       </c>
-      <c r="K21" s="68">
+      <c r="K21" s="66">
         <v>6</v>
       </c>
-      <c r="L21" s="123">
+      <c r="L21" s="121">
         <v>1</v>
       </c>
-      <c r="M21" s="65">
+      <c r="M21" s="63">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N21" s="152" t="s">
+      <c r="N21" s="150" t="s">
         <v>16</v>
       </c>
-      <c r="O21" s="66">
+      <c r="O21" s="64">
         <v>4.1349999999999998</v>
       </c>
-      <c r="P21" s="67">
+      <c r="P21" s="65">
         <f t="shared" si="1"/>
         <v>24.81</v>
       </c>
@@ -3225,48 +3263,48 @@
       <c r="A22" s="6">
         <v>20</v>
       </c>
-      <c r="B22" s="192"/>
-      <c r="C22" s="143" t="s">
+      <c r="B22" s="181"/>
+      <c r="C22" s="141" t="s">
+        <v>109</v>
+      </c>
+      <c r="D22" s="142" t="s">
+        <v>110</v>
+      </c>
+      <c r="E22" s="143" t="s">
+        <v>147</v>
+      </c>
+      <c r="F22" s="143" t="s">
         <v>111</v>
       </c>
-      <c r="D22" s="144" t="s">
-        <v>112</v>
-      </c>
-      <c r="E22" s="145" t="s">
-        <v>150</v>
-      </c>
-      <c r="F22" s="145" t="s">
-        <v>113</v>
-      </c>
-      <c r="G22" s="100" t="s">
-        <v>151</v>
-      </c>
-      <c r="H22" s="100" t="s">
-        <v>152</v>
-      </c>
-      <c r="I22" s="100" t="s">
+      <c r="G22" s="98" t="s">
+        <v>148</v>
+      </c>
+      <c r="H22" s="98" t="s">
+        <v>149</v>
+      </c>
+      <c r="I22" s="98" t="s">
         <v>39</v>
       </c>
-      <c r="J22" s="100" t="s">
+      <c r="J22" s="98" t="s">
         <v>22</v>
       </c>
-      <c r="K22" s="97">
+      <c r="K22" s="95">
         <v>10</v>
       </c>
-      <c r="L22" s="153">
+      <c r="L22" s="151">
         <v>1</v>
       </c>
-      <c r="M22" s="87">
+      <c r="M22" s="85">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N22" s="154" t="s">
+      <c r="N22" s="152" t="s">
         <v>16</v>
       </c>
-      <c r="O22" s="102">
+      <c r="O22" s="100">
         <v>5.8799999999999998E-2</v>
       </c>
-      <c r="P22" s="89">
+      <c r="P22" s="87">
         <f t="shared" si="1"/>
         <v>0.58799999999999997</v>
       </c>
@@ -3278,50 +3316,50 @@
       <c r="A23" s="6">
         <v>21</v>
       </c>
-      <c r="B23" s="190" t="s">
-        <v>120</v>
-      </c>
-      <c r="C23" s="140" t="s">
-        <v>115</v>
-      </c>
-      <c r="D23" s="141" t="s">
+      <c r="B23" s="179" t="s">
+        <v>117</v>
+      </c>
+      <c r="C23" s="138" t="s">
+        <v>113</v>
+      </c>
+      <c r="D23" s="139" t="s">
         <v>41</v>
       </c>
-      <c r="E23" s="116" t="s">
+      <c r="E23" s="114" t="s">
         <v>28</v>
       </c>
-      <c r="F23" s="147" t="s">
-        <v>116</v>
-      </c>
-      <c r="G23" s="58" t="s">
-        <v>153</v>
-      </c>
-      <c r="H23" s="58" t="s">
-        <v>154</v>
-      </c>
-      <c r="I23" s="57" t="s">
+      <c r="F23" s="145" t="s">
+        <v>114</v>
+      </c>
+      <c r="G23" s="56" t="s">
+        <v>150</v>
+      </c>
+      <c r="H23" s="56" t="s">
+        <v>151</v>
+      </c>
+      <c r="I23" s="55" t="s">
         <v>39</v>
       </c>
-      <c r="J23" s="57" t="s">
+      <c r="J23" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="K23" s="107">
+      <c r="K23" s="105">
         <v>50</v>
       </c>
-      <c r="L23" s="108">
+      <c r="L23" s="106">
         <v>1</v>
       </c>
-      <c r="M23" s="58">
+      <c r="M23" s="56">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N23" s="155" t="s">
+      <c r="N23" s="153" t="s">
         <v>16</v>
       </c>
-      <c r="O23" s="59">
+      <c r="O23" s="57">
         <v>1.5699999999999999E-2</v>
       </c>
-      <c r="P23" s="60">
+      <c r="P23" s="58">
         <f t="shared" si="1"/>
         <v>0.78499999999999992</v>
       </c>
@@ -3333,48 +3371,48 @@
       <c r="A24" s="6">
         <v>22</v>
       </c>
-      <c r="B24" s="191"/>
-      <c r="C24" s="151" t="s">
-        <v>168</v>
-      </c>
-      <c r="D24" s="125" t="s">
+      <c r="B24" s="180"/>
+      <c r="C24" s="149" t="s">
+        <v>165</v>
+      </c>
+      <c r="D24" s="123" t="s">
         <v>42</v>
       </c>
-      <c r="E24" s="121" t="s">
+      <c r="E24" s="119" t="s">
         <v>28</v>
       </c>
-      <c r="F24" s="121" t="s">
+      <c r="F24" s="119" t="s">
+        <v>164</v>
+      </c>
+      <c r="G24" s="62" t="s">
         <v>167</v>
       </c>
-      <c r="G24" s="64" t="s">
-        <v>170</v>
-      </c>
-      <c r="H24" s="64" t="s">
-        <v>169</v>
-      </c>
-      <c r="I24" s="64" t="s">
+      <c r="H24" s="62" t="s">
+        <v>166</v>
+      </c>
+      <c r="I24" s="62" t="s">
         <v>39</v>
       </c>
-      <c r="J24" s="64" t="s">
+      <c r="J24" s="62" t="s">
         <v>22</v>
       </c>
-      <c r="K24" s="64">
+      <c r="K24" s="62">
         <v>6</v>
       </c>
-      <c r="L24" s="109">
+      <c r="L24" s="107">
         <v>1</v>
       </c>
-      <c r="M24" s="65">
+      <c r="M24" s="63">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N24" s="194" t="s">
+      <c r="N24" s="169" t="s">
         <v>16</v>
       </c>
-      <c r="O24" s="106">
+      <c r="O24" s="104">
         <v>0.25409999999999999</v>
       </c>
-      <c r="P24" s="67">
+      <c r="P24" s="65">
         <f t="shared" si="1"/>
         <v>1.5246</v>
       </c>
@@ -3386,48 +3424,48 @@
       <c r="A25" s="6">
         <v>23</v>
       </c>
-      <c r="B25" s="191"/>
-      <c r="C25" s="151" t="s">
-        <v>117</v>
-      </c>
-      <c r="D25" s="125" t="s">
+      <c r="B25" s="180"/>
+      <c r="C25" s="149" t="s">
+        <v>115</v>
+      </c>
+      <c r="D25" s="123" t="s">
         <v>34</v>
       </c>
-      <c r="E25" s="121" t="s">
+      <c r="E25" s="119" t="s">
         <v>28</v>
       </c>
-      <c r="F25" s="156" t="s">
-        <v>118</v>
-      </c>
-      <c r="G25" s="64" t="s">
-        <v>155</v>
-      </c>
-      <c r="H25" s="64" t="s">
-        <v>156</v>
-      </c>
-      <c r="I25" s="64" t="s">
-        <v>161</v>
-      </c>
-      <c r="J25" s="64" t="s">
+      <c r="F25" s="154" t="s">
+        <v>116</v>
+      </c>
+      <c r="G25" s="62" t="s">
+        <v>152</v>
+      </c>
+      <c r="H25" s="62" t="s">
+        <v>153</v>
+      </c>
+      <c r="I25" s="62" t="s">
+        <v>158</v>
+      </c>
+      <c r="J25" s="62" t="s">
         <v>22</v>
       </c>
-      <c r="K25" s="64">
+      <c r="K25" s="62">
         <v>50</v>
       </c>
-      <c r="L25" s="109">
+      <c r="L25" s="107">
         <v>1</v>
       </c>
-      <c r="M25" s="65">
+      <c r="M25" s="63">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N25" s="152" t="s">
+      <c r="N25" s="150" t="s">
         <v>16</v>
       </c>
-      <c r="O25" s="66">
+      <c r="O25" s="64">
         <v>1.26E-2</v>
       </c>
-      <c r="P25" s="67">
+      <c r="P25" s="65">
         <f t="shared" si="1"/>
         <v>0.63</v>
       </c>
@@ -3435,157 +3473,193 @@
       <c r="R25" s="15"/>
       <c r="S25" s="11"/>
     </row>
-    <row r="26" spans="1:19" ht="90" thickBot="1">
+    <row r="26" spans="1:19" ht="102.75" thickBot="1">
       <c r="A26" s="19">
         <v>24</v>
       </c>
-      <c r="B26" s="191"/>
-      <c r="C26" s="157" t="s">
+      <c r="B26" s="180"/>
+      <c r="C26" s="155" t="s">
         <v>35</v>
       </c>
-      <c r="D26" s="158" t="s">
-        <v>119</v>
-      </c>
-      <c r="E26" s="159" t="s">
+      <c r="D26" s="156" t="s">
+        <v>170</v>
+      </c>
+      <c r="E26" s="157" t="s">
         <v>36</v>
       </c>
-      <c r="F26" s="159" t="s">
+      <c r="F26" s="157" t="s">
         <v>36</v>
       </c>
-      <c r="G26" s="110" t="s">
-        <v>157</v>
-      </c>
-      <c r="H26" s="110" t="s">
-        <v>157</v>
-      </c>
-      <c r="I26" s="111" t="s">
+      <c r="G26" s="108" t="s">
+        <v>154</v>
+      </c>
+      <c r="H26" s="108" t="s">
+        <v>154</v>
+      </c>
+      <c r="I26" s="109" t="s">
         <v>40</v>
       </c>
-      <c r="J26" s="111" t="s">
+      <c r="J26" s="109" t="s">
         <v>40</v>
       </c>
-      <c r="K26" s="112" t="s">
-        <v>157</v>
-      </c>
-      <c r="L26" s="113">
-        <v>42</v>
-      </c>
-      <c r="M26" s="114">
+      <c r="K26" s="110" t="s">
+        <v>154</v>
+      </c>
+      <c r="L26" s="111">
+        <v>47</v>
+      </c>
+      <c r="M26" s="112">
         <f t="shared" si="0"/>
-        <v>210</v>
-      </c>
-      <c r="N26" s="110" t="s">
-        <v>157</v>
-      </c>
-      <c r="O26" s="111" t="s">
+        <v>235</v>
+      </c>
+      <c r="N26" s="108" t="s">
+        <v>154</v>
+      </c>
+      <c r="O26" s="109" t="s">
         <v>40</v>
       </c>
-      <c r="P26" s="112" t="s">
-        <v>157</v>
+      <c r="P26" s="110" t="s">
+        <v>154</v>
       </c>
       <c r="Q26" s="45" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="R26" s="46"/>
       <c r="S26" s="11"/>
     </row>
     <row r="27" spans="1:19" ht="15.75" thickBot="1">
-      <c r="A27" s="19">
+      <c r="A27" s="19"/>
+      <c r="B27" s="189" t="s">
+        <v>161</v>
+      </c>
+      <c r="C27" s="198" t="s">
+        <v>174</v>
+      </c>
+      <c r="D27" s="194" t="s">
+        <v>40</v>
+      </c>
+      <c r="E27" s="194" t="s">
+        <v>40</v>
+      </c>
+      <c r="F27" s="194" t="s">
+        <v>40</v>
+      </c>
+      <c r="G27" s="194" t="s">
+        <v>40</v>
+      </c>
+      <c r="H27" s="194" t="s">
+        <v>40</v>
+      </c>
+      <c r="I27" s="194" t="s">
+        <v>40</v>
+      </c>
+      <c r="J27" s="194" t="s">
+        <v>40</v>
+      </c>
+      <c r="K27" s="194" t="s">
+        <v>40</v>
+      </c>
+      <c r="L27" s="194" t="s">
+        <v>40</v>
+      </c>
+      <c r="M27" s="194" t="s">
+        <v>40</v>
+      </c>
+      <c r="N27" s="194" t="s">
+        <v>40</v>
+      </c>
+      <c r="O27" s="194" t="s">
+        <v>40</v>
+      </c>
+      <c r="P27" s="194" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q27" s="195" t="s">
+        <v>159</v>
+      </c>
+      <c r="R27" s="182"/>
+      <c r="S27" s="11"/>
+    </row>
+    <row r="28" spans="1:19" ht="15.75" thickBot="1">
+      <c r="A28" s="19">
         <v>25</v>
       </c>
-      <c r="B27" s="160" t="s">
-        <v>164</v>
-      </c>
-      <c r="C27" s="171" t="s">
-        <v>165</v>
-      </c>
-      <c r="D27" s="178" t="s">
+      <c r="B28" s="190"/>
+      <c r="C28" s="196" t="s">
+        <v>172</v>
+      </c>
+      <c r="D28" s="183" t="s">
         <v>40</v>
       </c>
-      <c r="E27" s="178" t="s">
+      <c r="E28" s="183" t="s">
         <v>40</v>
       </c>
-      <c r="F27" s="172" t="s">
-        <v>165</v>
-      </c>
-      <c r="G27" s="178" t="s">
+      <c r="F28" s="183" t="s">
+        <v>162</v>
+      </c>
+      <c r="G28" s="183" t="s">
+        <v>173</v>
+      </c>
+      <c r="H28" s="183" t="s">
         <v>40</v>
       </c>
-      <c r="H27" s="178" t="s">
+      <c r="I28" s="183" t="s">
         <v>40</v>
       </c>
-      <c r="I27" s="178" t="s">
+      <c r="J28" s="183" t="s">
         <v>40</v>
       </c>
-      <c r="J27" s="178" t="s">
+      <c r="K28" s="183" t="s">
         <v>40</v>
       </c>
-      <c r="K27" s="178" t="s">
-        <v>40</v>
-      </c>
-      <c r="L27" s="175">
+      <c r="L28" s="184">
         <v>1</v>
       </c>
-      <c r="M27" s="175">
+      <c r="M28" s="184">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N27" s="173"/>
-      <c r="O27" s="174"/>
-      <c r="P27" s="174"/>
-      <c r="Q27" s="176"/>
-      <c r="R27" s="177"/>
-      <c r="S27" s="11"/>
-    </row>
-    <row r="28" spans="1:19" ht="15.75">
-      <c r="A28" s="1"/>
-      <c r="C28" s="25"/>
-      <c r="D28" s="8"/>
-      <c r="E28" s="7"/>
-      <c r="G28" s="7"/>
-      <c r="H28" s="7"/>
-      <c r="I28" s="7"/>
-      <c r="J28" s="7"/>
-      <c r="K28" s="7"/>
-      <c r="L28" s="186" t="s">
-        <v>37</v>
-      </c>
-      <c r="M28" s="187"/>
-      <c r="N28" s="187"/>
-      <c r="O28" s="51"/>
-      <c r="P28" s="52">
-        <f>SUM(P3:P26)</f>
-        <v>248.20189999999997</v>
-      </c>
-      <c r="Q28" s="7"/>
-      <c r="R28" s="7"/>
+      <c r="N28" s="185" t="s">
+        <v>171</v>
+      </c>
+      <c r="O28" s="186">
+        <v>3.35</v>
+      </c>
+      <c r="P28" s="187">
+        <f>O28*M28</f>
+        <v>16.75</v>
+      </c>
+      <c r="Q28" s="197" t="s">
+        <v>159</v>
+      </c>
+      <c r="R28" s="188"/>
       <c r="S28" s="11"/>
     </row>
-    <row r="29" spans="1:19" ht="16.5" thickBot="1">
+    <row r="29" spans="1:19" ht="15.75">
       <c r="A29" s="1"/>
       <c r="C29" s="25"/>
-      <c r="E29" s="29"/>
-      <c r="F29" s="29"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="7"/>
       <c r="G29" s="7"/>
       <c r="H29" s="7"/>
       <c r="I29" s="7"/>
       <c r="J29" s="7"/>
       <c r="K29" s="7"/>
-      <c r="L29" s="188" t="s">
-        <v>38</v>
-      </c>
-      <c r="M29" s="189"/>
-      <c r="N29" s="189"/>
-      <c r="O29" s="48"/>
-      <c r="P29" s="53">
-        <f>P28/5</f>
-        <v>49.640379999999993</v>
+      <c r="L29" s="191" t="s">
+        <v>37</v>
+      </c>
+      <c r="M29" s="192"/>
+      <c r="N29" s="192"/>
+      <c r="O29" s="21"/>
+      <c r="P29" s="193">
+        <f>SUM(P3:P28)</f>
+        <v>264.95189999999997</v>
       </c>
       <c r="Q29" s="7"/>
       <c r="R29" s="7"/>
       <c r="S29" s="11"/>
     </row>
-    <row r="30" spans="1:19" ht="15.75">
+    <row r="30" spans="1:19" ht="16.5" thickBot="1">
       <c r="A30" s="1"/>
       <c r="C30" s="25"/>
       <c r="E30" s="29"/>
@@ -3595,57 +3669,79 @@
       <c r="I30" s="7"/>
       <c r="J30" s="7"/>
       <c r="K30" s="7"/>
-      <c r="L30" s="38"/>
-      <c r="M30" s="179" t="s">
-        <v>160</v>
-      </c>
-      <c r="N30" s="180"/>
-      <c r="O30" s="39"/>
-      <c r="P30" s="50"/>
+      <c r="L30" s="177" t="s">
+        <v>38</v>
+      </c>
+      <c r="M30" s="178"/>
+      <c r="N30" s="178"/>
+      <c r="O30" s="199">
+        <f>SUM(O3:O28)</f>
+        <v>31.2363</v>
+      </c>
+      <c r="P30" s="51">
+        <f>P29/5</f>
+        <v>52.990379999999995</v>
+      </c>
       <c r="Q30" s="7"/>
       <c r="R30" s="7"/>
       <c r="S30" s="11"/>
     </row>
     <row r="31" spans="1:19" ht="15.75">
       <c r="A31" s="1"/>
-      <c r="D31" s="28"/>
+      <c r="C31" s="25"/>
       <c r="E31" s="29"/>
-      <c r="M31" s="179" t="s">
+      <c r="F31" s="29"/>
+      <c r="G31" s="7"/>
+      <c r="H31" s="7"/>
+      <c r="I31" s="7"/>
+      <c r="J31" s="7"/>
+      <c r="K31" s="7"/>
+      <c r="L31" s="38"/>
+      <c r="M31" s="170" t="s">
+        <v>157</v>
+      </c>
+      <c r="N31" s="171"/>
+      <c r="O31" s="39"/>
+      <c r="P31" s="50"/>
+      <c r="Q31" s="7"/>
+      <c r="R31" s="7"/>
+      <c r="S31" s="11"/>
+    </row>
+    <row r="32" spans="1:19" ht="15.75">
+      <c r="A32" s="1"/>
+      <c r="D32" s="28"/>
+      <c r="E32" s="29"/>
+      <c r="M32" s="170" t="s">
         <v>43</v>
       </c>
-      <c r="N31" s="180"/>
-      <c r="O31" s="21"/>
-      <c r="P31" s="47">
+      <c r="N32" s="171"/>
+      <c r="O32" s="21"/>
+      <c r="P32" s="47">
         <v>213.77</v>
-      </c>
-      <c r="R31" s="11"/>
-      <c r="S31" s="11"/>
-    </row>
-    <row r="32" spans="1:19" ht="16.5" thickBot="1">
-      <c r="A32" s="1"/>
-      <c r="D32" s="29"/>
-      <c r="M32" s="181" t="s">
-        <v>44</v>
-      </c>
-      <c r="N32" s="182"/>
-      <c r="O32" s="48"/>
-      <c r="P32" s="49">
-        <f>P31+P28</f>
-        <v>461.97190000000001</v>
       </c>
       <c r="R32" s="11"/>
       <c r="S32" s="11"/>
     </row>
-    <row r="33" spans="1:19">
+    <row r="33" spans="1:19" ht="16.5" thickBot="1">
       <c r="A33" s="1"/>
-      <c r="C33" s="26"/>
       <c r="D33" s="29"/>
-      <c r="M33" s="20"/>
+      <c r="M33" s="172" t="s">
+        <v>44</v>
+      </c>
+      <c r="N33" s="173"/>
+      <c r="O33" s="48"/>
+      <c r="P33" s="49">
+        <f>P32+P29</f>
+        <v>478.72190000000001</v>
+      </c>
       <c r="R33" s="11"/>
       <c r="S33" s="11"/>
     </row>
     <row r="34" spans="1:19">
       <c r="A34" s="1"/>
+      <c r="C34" s="26"/>
+      <c r="D34" s="29"/>
+      <c r="M34" s="20"/>
       <c r="R34" s="11"/>
       <c r="S34" s="11"/>
     </row>
@@ -3664,12 +3760,12 @@
       <c r="R37" s="11"/>
       <c r="S37" s="11"/>
     </row>
-    <row r="38" spans="1:19" ht="15.75" customHeight="1">
+    <row r="38" spans="1:19">
       <c r="A38" s="1"/>
       <c r="R38" s="11"/>
       <c r="S38" s="11"/>
     </row>
-    <row r="39" spans="1:19">
+    <row r="39" spans="1:19" ht="15.75" customHeight="1">
       <c r="A39" s="1"/>
       <c r="R39" s="11"/>
       <c r="S39" s="11"/>
@@ -3695,26 +3791,32 @@
       <c r="S43" s="11"/>
     </row>
     <row r="44" spans="1:19">
-      <c r="H44" s="9"/>
-      <c r="Q44" s="10"/>
+      <c r="A44" s="1"/>
+      <c r="R44" s="11"/>
+      <c r="S44" s="11"/>
     </row>
     <row r="45" spans="1:19">
       <c r="H45" s="9"/>
       <c r="Q45" s="10"/>
     </row>
+    <row r="46" spans="1:19">
+      <c r="H46" s="9"/>
+      <c r="Q46" s="10"/>
+    </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="M30:N30"/>
+  <mergeCells count="12">
     <mergeCell ref="M31:N31"/>
     <mergeCell ref="M32:N32"/>
+    <mergeCell ref="M33:N33"/>
     <mergeCell ref="A1:R1"/>
-    <mergeCell ref="L28:N28"/>
     <mergeCell ref="L29:N29"/>
+    <mergeCell ref="L30:N30"/>
     <mergeCell ref="B3:B10"/>
     <mergeCell ref="B13:B14"/>
     <mergeCell ref="B15:B16"/>
     <mergeCell ref="B17:B22"/>
     <mergeCell ref="B23:B26"/>
+    <mergeCell ref="B27:B28"/>
   </mergeCells>
   <phoneticPr fontId="16" type="noConversion"/>
   <conditionalFormatting sqref="Q24">
@@ -3771,7 +3873,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P29:P30">
+  <conditionalFormatting sqref="P30:P31">
     <cfRule type="dataBar" priority="28">
       <dataBar>
         <cfvo type="min"/>
@@ -3785,7 +3887,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L17:M27 L8:L14 M3:M27">
+  <conditionalFormatting sqref="L17:M26 L8:L14 M3:M26 L28:M28">
     <cfRule type="colorScale" priority="30">
       <colorScale>
         <cfvo type="min"/>
@@ -3797,7 +3899,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L3:M27">
+  <conditionalFormatting sqref="L3:M26 L28:M28">
     <cfRule type="colorScale" priority="33">
       <colorScale>
         <cfvo type="min"/>
@@ -3809,7 +3911,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P3:P27">
+  <conditionalFormatting sqref="P3:P26 P28">
     <cfRule type="dataBar" priority="34">
       <dataBar>
         <cfvo type="min"/>
@@ -3838,28 +3940,28 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="N3" r:id="rId1" xr:uid="{77E7F02B-CC4A-45E7-B730-3717F029D629}"/>
-    <hyperlink ref="N4" r:id="rId2" xr:uid="{422ACB32-99A4-4373-9BBC-0F8302D669E9}"/>
-    <hyperlink ref="N5" r:id="rId3" xr:uid="{1D3C339F-D2BF-414A-BD64-13F776D76A9F}"/>
-    <hyperlink ref="N6" r:id="rId4" xr:uid="{01BBFB8E-A26B-48C7-AB0F-DF9F65C47B93}"/>
-    <hyperlink ref="N7" r:id="rId5" xr:uid="{83C85DDA-7FBA-4A9B-8C90-61DA15EF09A1}"/>
-    <hyperlink ref="N8" r:id="rId6" xr:uid="{F5D2937B-2705-425B-A920-F69EE337A9AA}"/>
-    <hyperlink ref="N9" r:id="rId7" xr:uid="{23650E7E-1F91-465B-A508-B3E81A5A29DB}"/>
-    <hyperlink ref="N10" r:id="rId8" xr:uid="{A3FA0792-9C1C-4B11-8EC7-D8950B40778A}"/>
-    <hyperlink ref="N12" r:id="rId9" xr:uid="{9306F7E1-9FA0-45C1-9226-A5EFFE620B9F}"/>
-    <hyperlink ref="N13" r:id="rId10" xr:uid="{6C2F24FA-F4C6-4765-90C1-BBDF944038A7}"/>
-    <hyperlink ref="N14" r:id="rId11" xr:uid="{834B4123-1D60-4B34-B015-5E7BBC8F47AF}"/>
-    <hyperlink ref="N15" r:id="rId12" xr:uid="{1D1A071F-2A3D-4FA1-937C-5E9315A2DAC9}"/>
-    <hyperlink ref="N16" r:id="rId13" xr:uid="{1ECC2B27-3B6B-4070-A52B-CBF10AA116AF}"/>
-    <hyperlink ref="N17" r:id="rId14" xr:uid="{BFDF2136-290A-40AE-829A-CE2FE24D8034}"/>
-    <hyperlink ref="N18" r:id="rId15" xr:uid="{E71028CE-6136-4648-ABFC-ABDBCFA60DB5}"/>
-    <hyperlink ref="N19" r:id="rId16" xr:uid="{600C5A90-1D13-491E-82D2-49A3F9B676E0}"/>
-    <hyperlink ref="N21" r:id="rId17" xr:uid="{F5B5F1A9-E737-48E7-A459-388501647F5A}"/>
-    <hyperlink ref="N22" r:id="rId18" xr:uid="{8E22EBA9-5C52-408B-A65B-4F115F1CD0F7}"/>
-    <hyperlink ref="N23" r:id="rId19" xr:uid="{0A7E773D-5A3D-486C-84CA-8D29060909A3}"/>
-    <hyperlink ref="N25" r:id="rId20" xr:uid="{79B90123-86F4-4C7F-BE0B-E5B7C590F601}"/>
-    <hyperlink ref="N11" r:id="rId21" display="Aliexpress" xr:uid="{D571A1A4-A3B8-476C-81AA-A10E0576C945}"/>
-    <hyperlink ref="N24" r:id="rId22" xr:uid="{552B4167-57FF-43F1-B0A5-FDF3A29237A4}"/>
+    <hyperlink ref="N3" r:id="rId1"/>
+    <hyperlink ref="N4" r:id="rId2"/>
+    <hyperlink ref="N5" r:id="rId3"/>
+    <hyperlink ref="N6" r:id="rId4"/>
+    <hyperlink ref="N7" r:id="rId5"/>
+    <hyperlink ref="N8" r:id="rId6"/>
+    <hyperlink ref="N9" r:id="rId7"/>
+    <hyperlink ref="N10" r:id="rId8"/>
+    <hyperlink ref="N12" r:id="rId9"/>
+    <hyperlink ref="N13" r:id="rId10"/>
+    <hyperlink ref="N14" r:id="rId11"/>
+    <hyperlink ref="N15" r:id="rId12"/>
+    <hyperlink ref="N16" r:id="rId13"/>
+    <hyperlink ref="N17" r:id="rId14"/>
+    <hyperlink ref="N18" r:id="rId15"/>
+    <hyperlink ref="N19" r:id="rId16"/>
+    <hyperlink ref="N21" r:id="rId17"/>
+    <hyperlink ref="N22" r:id="rId18"/>
+    <hyperlink ref="N23" r:id="rId19"/>
+    <hyperlink ref="N25" r:id="rId20"/>
+    <hyperlink ref="N11" r:id="rId21" display="Aliexpress"/>
+    <hyperlink ref="N24" r:id="rId22"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId23"/>
@@ -3916,7 +4018,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>P29:P30</xm:sqref>
+          <xm:sqref>P30:P31</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{70CE0387-EDB2-443C-842F-1D5EE6E70AF7}">
@@ -3929,7 +4031,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>P3:P27</xm:sqref>
+          <xm:sqref>P3:P26 P28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{193AFC57-9059-4DAB-9E2A-67F7DD9723ED}">

</xml_diff>